<commit_message>
Dash Canguru + Atualizacao
</commit_message>
<xml_diff>
--- a/Bases/Navegacao_Menu.xlsx
+++ b/Bases/Navegacao_Menu.xlsx
@@ -1,19 +1,20 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28925"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29231"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\djdan\Documents\GitHub\Dash-Upmat\Bases\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0190EFB3-D59E-42F9-A6B6-312F72243BB9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B9DF9C49-BD03-4371-9A81-F8C18D46CF14}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="23880" yWindow="510" windowWidth="20730" windowHeight="11040" xr2:uid="{F34CCB2F-E2D2-4F06-83D1-8921BB237BC6}"/>
+    <workbookView xWindow="23880" yWindow="855" windowWidth="20640" windowHeight="11040" activeTab="1" xr2:uid="{F34CCB2F-E2D2-4F06-83D1-8921BB237BC6}"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="2" r:id="rId1"/>
+    <sheet name="Olitef" sheetId="2" r:id="rId1"/>
+    <sheet name="Kangaroo" sheetId="3" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -36,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="107" uniqueCount="24">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="194" uniqueCount="32">
   <si>
     <t>Ordem</t>
   </si>
@@ -108,6 +109,30 @@
   </si>
   <si>
     <t>Listagem Prof x Estud</t>
+  </si>
+  <si>
+    <t>Respondentes</t>
+  </si>
+  <si>
+    <t>Inscrições 2026 - Part1</t>
+  </si>
+  <si>
+    <t>Inscrições 2026 - Part2</t>
+  </si>
+  <si>
+    <t>Busca Inscrições MKT 2026</t>
+  </si>
+  <si>
+    <t>Conversão 2026 - Part1</t>
+  </si>
+  <si>
+    <t>Conversão 2026 - Part2</t>
+  </si>
+  <si>
+    <t>Inscrições 2025</t>
+  </si>
+  <si>
+    <t>Busca Inscrições 2025</t>
   </si>
 </sst>
 </file>
@@ -497,7 +522,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{19030B0D-2A8E-4C3B-9DF6-B05FCD013344}">
-  <dimension ref="A1:C53"/>
+  <dimension ref="A1:C57"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="24.28515625" bestFit="1" customWidth="1"/>
@@ -828,10 +853,10 @@
         <v>9</v>
       </c>
       <c r="B30" s="1" t="s">
-        <v>17</v>
+        <v>24</v>
       </c>
       <c r="C30" s="1" t="s">
-        <v>6</v>
+        <v>19</v>
       </c>
     </row>
     <row r="31" spans="1:3" x14ac:dyDescent="0.25">
@@ -839,40 +864,40 @@
         <v>9</v>
       </c>
       <c r="B31" s="1" t="s">
-        <v>17</v>
+        <v>24</v>
       </c>
       <c r="C31" s="1" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="32" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A32" s="1">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B32" s="1" t="s">
-        <v>16</v>
+        <v>24</v>
       </c>
       <c r="C32" s="1" t="s">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="33" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A33" s="1">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B33" s="1" t="s">
-        <v>16</v>
+        <v>24</v>
       </c>
       <c r="C33" s="1" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="34" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A34" s="1">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B34" s="1" t="s">
-        <v>21</v>
+        <v>17</v>
       </c>
       <c r="C34" s="1" t="s">
         <v>6</v>
@@ -880,32 +905,32 @@
     </row>
     <row r="35" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A35" s="1">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B35" s="1" t="s">
-        <v>21</v>
+        <v>17</v>
       </c>
       <c r="C35" s="1" t="s">
-        <v>19</v>
+        <v>5</v>
       </c>
     </row>
     <row r="36" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A36" s="1">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B36" s="1" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="C36" s="1" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
     </row>
     <row r="37" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A37" s="1">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B37" s="1" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="C37" s="1" t="s">
         <v>5</v>
@@ -913,46 +938,46 @@
     </row>
     <row r="38" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A38" s="1">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B38" s="1" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="C38" s="1" t="s">
-        <v>19</v>
+        <v>6</v>
       </c>
     </row>
     <row r="39" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A39" s="1">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B39" s="1" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="C39" s="1" t="s">
-        <v>6</v>
+        <v>19</v>
       </c>
     </row>
     <row r="40" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A40" s="1">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B40" s="1" t="s">
-        <v>12</v>
+        <v>18</v>
       </c>
       <c r="C40" s="1" t="s">
-        <v>19</v>
+        <v>6</v>
       </c>
     </row>
     <row r="41" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A41" s="1">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B41" s="1" t="s">
-        <v>12</v>
+        <v>18</v>
       </c>
       <c r="C41" s="1" t="s">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="42" spans="1:3" x14ac:dyDescent="0.25">
@@ -960,10 +985,10 @@
         <v>14</v>
       </c>
       <c r="B42" s="1" t="s">
-        <v>12</v>
+        <v>23</v>
       </c>
       <c r="C42" s="1" t="s">
-        <v>5</v>
+        <v>19</v>
       </c>
     </row>
     <row r="43" spans="1:3" x14ac:dyDescent="0.25">
@@ -971,7 +996,7 @@
         <v>14</v>
       </c>
       <c r="B43" s="1" t="s">
-        <v>12</v>
+        <v>23</v>
       </c>
       <c r="C43" s="1" t="s">
         <v>6</v>
@@ -982,7 +1007,7 @@
         <v>15</v>
       </c>
       <c r="B44" s="1" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C44" s="1" t="s">
         <v>19</v>
@@ -993,7 +1018,7 @@
         <v>15</v>
       </c>
       <c r="B45" s="1" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C45" s="1" t="s">
         <v>4</v>
@@ -1004,7 +1029,7 @@
         <v>15</v>
       </c>
       <c r="B46" s="1" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C46" s="1" t="s">
         <v>5</v>
@@ -1015,7 +1040,7 @@
         <v>15</v>
       </c>
       <c r="B47" s="1" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C47" s="1" t="s">
         <v>6</v>
@@ -1026,10 +1051,10 @@
         <v>16</v>
       </c>
       <c r="B48" s="1" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C48" s="1" t="s">
-        <v>4</v>
+        <v>19</v>
       </c>
     </row>
     <row r="49" spans="1:3" x14ac:dyDescent="0.25">
@@ -1037,10 +1062,10 @@
         <v>16</v>
       </c>
       <c r="B49" s="1" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C49" s="1" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="50" spans="1:3" x14ac:dyDescent="0.25">
@@ -1048,21 +1073,21 @@
         <v>16</v>
       </c>
       <c r="B50" s="1" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C50" s="1" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
     </row>
     <row r="51" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A51" s="1">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B51" s="1" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="C51" s="1" t="s">
-        <v>4</v>
+        <v>6</v>
       </c>
     </row>
     <row r="52" spans="1:3" x14ac:dyDescent="0.25">
@@ -1070,10 +1095,10 @@
         <v>17</v>
       </c>
       <c r="B52" s="1" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C52" s="1" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="53" spans="1:3" x14ac:dyDescent="0.25">
@@ -1081,9 +1106,53 @@
         <v>17</v>
       </c>
       <c r="B53" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="C53" s="1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="54" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A54" s="1">
+        <v>17</v>
+      </c>
+      <c r="B54" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="C54" s="1" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="55" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A55" s="1">
+        <v>18</v>
+      </c>
+      <c r="B55" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="C53" s="1" t="s">
+      <c r="C55" s="1" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="56" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A56" s="1">
+        <v>18</v>
+      </c>
+      <c r="B56" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="C56" s="1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="57" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A57" s="1">
+        <v>18</v>
+      </c>
+      <c r="B57" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="C57" s="1" t="s">
         <v>6</v>
       </c>
     </row>
@@ -1094,4 +1163,447 @@
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C7F7F84F-51F4-4AA7-8488-D6CFB2C033F7}">
+  <dimension ref="A1:C39"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="2" max="2" width="24.28515625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="27.28515625" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A2" s="1">
+        <v>1</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A3" s="1">
+        <v>1</v>
+      </c>
+      <c r="B3" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="C3" s="1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A4" s="1">
+        <v>1</v>
+      </c>
+      <c r="B4" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="C4" s="1" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A5" s="1">
+        <v>2</v>
+      </c>
+      <c r="B5" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="C5" s="1" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A6" s="1">
+        <v>2</v>
+      </c>
+      <c r="B6" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="C6" s="1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A7" s="1">
+        <v>2</v>
+      </c>
+      <c r="B7" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="C7" s="1" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A8" s="1">
+        <v>3</v>
+      </c>
+      <c r="B8" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="C8" s="1" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A9" s="1">
+        <v>3</v>
+      </c>
+      <c r="B9" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="C9" s="1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A10" s="1">
+        <v>3</v>
+      </c>
+      <c r="B10" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="C10" s="1" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A11" s="1">
+        <v>4</v>
+      </c>
+      <c r="B11" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="C11" s="1" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A12" s="1">
+        <v>4</v>
+      </c>
+      <c r="B12" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="C12" s="1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A13" s="1">
+        <v>4</v>
+      </c>
+      <c r="B13" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="C13" s="1" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A14" s="1">
+        <v>5</v>
+      </c>
+      <c r="B14" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="C14" s="1" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="15" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A15" s="1">
+        <v>5</v>
+      </c>
+      <c r="B15" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="C15" s="1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="16" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A16" s="1">
+        <v>5</v>
+      </c>
+      <c r="B16" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="C16" s="1" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="17" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A17" s="1">
+        <v>6</v>
+      </c>
+      <c r="B17" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="C17" s="1" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="18" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A18" s="1">
+        <v>6</v>
+      </c>
+      <c r="B18" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="C18" s="1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="19" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A19" s="1">
+        <v>6</v>
+      </c>
+      <c r="B19" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="C19" s="1" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="20" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A20" s="1">
+        <v>7</v>
+      </c>
+      <c r="B20" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="C20" s="1" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="21" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A21" s="1">
+        <v>7</v>
+      </c>
+      <c r="B21" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="C21" s="1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="22" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A22" s="1">
+        <v>7</v>
+      </c>
+      <c r="B22" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="C22" s="1" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="23" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A23" s="1">
+        <v>8</v>
+      </c>
+      <c r="B23" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="C23" s="1" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="24" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A24" s="1">
+        <v>8</v>
+      </c>
+      <c r="B24" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="C24" s="1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="25" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A25" s="1">
+        <v>8</v>
+      </c>
+      <c r="B25" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="C25" s="1" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="26" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A26" s="1">
+        <v>9</v>
+      </c>
+      <c r="B26" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="C26" s="1" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="27" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A27" s="1">
+        <v>9</v>
+      </c>
+      <c r="B27" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="C27" s="1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="28" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A28" s="1">
+        <v>10</v>
+      </c>
+      <c r="B28" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="C28" s="1" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="29" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A29" s="1">
+        <v>10</v>
+      </c>
+      <c r="B29" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="C29" s="1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="30" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A30" s="1">
+        <v>10</v>
+      </c>
+      <c r="B30" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="C30" s="1" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="31" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A31" s="1">
+        <v>11</v>
+      </c>
+      <c r="B31" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="C31" s="1" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="32" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A32" s="1">
+        <v>11</v>
+      </c>
+      <c r="B32" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="C32" s="1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="33" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A33" s="1">
+        <v>11</v>
+      </c>
+      <c r="B33" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="C33" s="1" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="34" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A34" s="1">
+        <v>12</v>
+      </c>
+      <c r="B34" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="C34" s="1" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="35" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A35" s="1">
+        <v>12</v>
+      </c>
+      <c r="B35" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="C35" s="1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="36" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A36" s="1">
+        <v>12</v>
+      </c>
+      <c r="B36" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="C36" s="1" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="37" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A37" s="1">
+        <v>13</v>
+      </c>
+      <c r="B37" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="C37" s="1" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="38" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A38" s="1">
+        <v>13</v>
+      </c>
+      <c r="B38" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="C38" s="1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="39" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A39" s="1">
+        <v>13</v>
+      </c>
+      <c r="B39" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="C39" s="1" t="s">
+        <v>6</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Tela Seleção de Provas
</commit_message>
<xml_diff>
--- a/Bases/Navegacao_Menu.xlsx
+++ b/Bases/Navegacao_Menu.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29530"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\djdan\Documents\GitHub\Dash-Upmat\Bases\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E796461A-2BF6-47DE-AC7F-0D2695825A9B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3D076DE6-B4F6-4CCA-8193-FB1BB5C5D99B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="24240" windowHeight="13020" activeTab="1" xr2:uid="{F34CCB2F-E2D2-4F06-83D1-8921BB237BC6}"/>
   </bookViews>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="191" uniqueCount="43">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="197" uniqueCount="44">
   <si>
     <t>Ordem</t>
   </si>
@@ -151,9 +151,6 @@
     <t>Potencial de Conversão Inscrições 2025 - Part1</t>
   </si>
   <si>
-    <t>Listagem de Escolas Inscrições 2025 X 2026</t>
-  </si>
-  <si>
     <t>Migração Experience 2025 x 2026</t>
   </si>
   <si>
@@ -167,6 +164,12 @@
   </si>
   <si>
     <t>Listagem de Escolas Inscritas 2026</t>
+  </si>
+  <si>
+    <t>Listagem de Escolas Inscrições 2025</t>
+  </si>
+  <si>
+    <t>Seleção de Provas 2026</t>
   </si>
 </sst>
 </file>
@@ -1212,7 +1215,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C7F7F84F-51F4-4AA7-8488-D6CFB2C033F7}">
-  <dimension ref="A1:C32"/>
+  <dimension ref="A1:C35"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="42.5703125" bestFit="1" customWidth="1"/>
@@ -1301,7 +1304,7 @@
         <v>3</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="C8" s="1" t="s">
         <v>4</v>
@@ -1312,7 +1315,7 @@
         <v>3</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="C9" s="1" t="s">
         <v>6</v>
@@ -1323,7 +1326,7 @@
         <v>3</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="C10" s="1" t="s">
         <v>5</v>
@@ -1334,7 +1337,7 @@
         <v>4</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="C11" s="1" t="s">
         <v>4</v>
@@ -1345,10 +1348,10 @@
         <v>4</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="C12" s="1" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.25">
@@ -1356,10 +1359,10 @@
         <v>4</v>
       </c>
       <c r="B13" s="1" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="C13" s="1" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.25">
@@ -1403,7 +1406,7 @@
         <v>39</v>
       </c>
       <c r="C17" s="1" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.25">
@@ -1425,7 +1428,7 @@
         <v>39</v>
       </c>
       <c r="C19" s="1" t="s">
-        <v>4</v>
+        <v>6</v>
       </c>
     </row>
     <row r="20" spans="1:3" x14ac:dyDescent="0.25">
@@ -1436,7 +1439,7 @@
         <v>38</v>
       </c>
       <c r="C20" s="1" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="21" spans="1:3" x14ac:dyDescent="0.25">
@@ -1447,7 +1450,7 @@
         <v>38</v>
       </c>
       <c r="C21" s="1" t="s">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="22" spans="1:3" x14ac:dyDescent="0.25">
@@ -1458,7 +1461,7 @@
         <v>38</v>
       </c>
       <c r="C22" s="1" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
     </row>
     <row r="23" spans="1:3" x14ac:dyDescent="0.25">
@@ -1466,29 +1469,29 @@
         <v>8</v>
       </c>
       <c r="B23" s="1" t="s">
-        <v>27</v>
+        <v>37</v>
       </c>
       <c r="C23" s="1" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
     </row>
     <row r="24" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A24" s="1">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B24" s="1" t="s">
         <v>37</v>
       </c>
       <c r="C24" s="1" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
     </row>
     <row r="25" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A25" s="1">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="B25" s="1" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="C25" s="1" t="s">
         <v>6</v>
@@ -1496,10 +1499,10 @@
     </row>
     <row r="26" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A26" s="1">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="B26" s="1" t="s">
-        <v>35</v>
+        <v>27</v>
       </c>
       <c r="C26" s="1" t="s">
         <v>6</v>
@@ -1507,10 +1510,10 @@
     </row>
     <row r="27" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A27" s="1">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="B27" s="1" t="s">
-        <v>34</v>
+        <v>42</v>
       </c>
       <c r="C27" s="1" t="s">
         <v>6</v>
@@ -1518,10 +1521,10 @@
     </row>
     <row r="28" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A28" s="1">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="B28" s="1" t="s">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="C28" s="1" t="s">
         <v>6</v>
@@ -1529,10 +1532,10 @@
     </row>
     <row r="29" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A29" s="1">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="B29" s="1" t="s">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="C29" s="1" t="s">
         <v>6</v>
@@ -1540,10 +1543,10 @@
     </row>
     <row r="30" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A30" s="1">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="B30" s="1" t="s">
-        <v>31</v>
+        <v>34</v>
       </c>
       <c r="C30" s="1" t="s">
         <v>6</v>
@@ -1551,10 +1554,10 @@
     </row>
     <row r="31" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A31" s="1">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="B31" s="1" t="s">
-        <v>29</v>
+        <v>33</v>
       </c>
       <c r="C31" s="1" t="s">
         <v>6</v>
@@ -1562,12 +1565,45 @@
     </row>
     <row r="32" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A32" s="1">
+        <v>15</v>
+      </c>
+      <c r="B32" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="C32" s="1" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="33" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A33" s="1">
+        <v>16</v>
+      </c>
+      <c r="B33" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="C33" s="1" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="34" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A34" s="1">
         <v>17</v>
       </c>
-      <c r="B32" t="s">
+      <c r="B34" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="C34" s="1" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="35" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A35" s="1">
+        <v>18</v>
+      </c>
+      <c r="B35" t="s">
         <v>30</v>
       </c>
-      <c r="C32" s="1" t="s">
+      <c r="C35" s="1" t="s">
         <v>6</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Melhorias B3 + Canguru
</commit_message>
<xml_diff>
--- a/Bases/Navegacao_Menu.xlsx
+++ b/Bases/Navegacao_Menu.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\djdan\Documents\GitHub\Dash-Upmat\Bases\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{20777F3A-2EAA-4075-96DA-A0C41DFB369B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AA80270D-1EA3-4985-B024-249E7D277F98}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="24240" windowHeight="13020" activeTab="3" xr2:uid="{F34CCB2F-E2D2-4F06-83D1-8921BB237BC6}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="364" uniqueCount="53">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="372" uniqueCount="54">
   <si>
     <t>Ordem</t>
   </si>
@@ -198,6 +198,9 @@
   </si>
   <si>
     <t>Listagem de Escolas Inscritas 2026 (B3)</t>
+  </si>
+  <si>
+    <t>Alcance nas Cidades</t>
   </si>
 </sst>
 </file>
@@ -248,11 +251,10 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -2203,7 +2205,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7F446C31-FA66-4630-B110-19ECB8E7DF76}">
-  <dimension ref="A1:C37"/>
+  <dimension ref="A1:C41"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="42.5703125" bestFit="1" customWidth="1"/>
@@ -2228,7 +2230,7 @@
       <c r="B2" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="C2" s="3" t="s">
+      <c r="C2" t="s">
         <v>19</v>
       </c>
     </row>
@@ -2272,7 +2274,7 @@
       <c r="B6" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="C6" s="3" t="s">
+      <c r="C6" t="s">
         <v>19</v>
       </c>
     </row>
@@ -2501,40 +2503,40 @@
         <v>8</v>
       </c>
       <c r="B27" s="1" t="s">
-        <v>20</v>
+        <v>53</v>
       </c>
       <c r="C27" s="1" t="s">
-        <v>6</v>
+        <v>19</v>
       </c>
     </row>
     <row r="28" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A28" s="1">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B28" s="1" t="s">
-        <v>24</v>
+        <v>53</v>
       </c>
       <c r="C28" s="1" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
     </row>
     <row r="29" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A29" s="1">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="B29" s="1" t="s">
-        <v>17</v>
+        <v>53</v>
       </c>
       <c r="C29" s="1" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
     </row>
     <row r="30" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A30" s="1">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="B30" s="1" t="s">
-        <v>16</v>
+        <v>53</v>
       </c>
       <c r="C30" s="1" t="s">
         <v>6</v>
@@ -2542,10 +2544,10 @@
     </row>
     <row r="31" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A31" s="1">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="B31" s="1" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="C31" s="1" t="s">
         <v>6</v>
@@ -2553,10 +2555,10 @@
     </row>
     <row r="32" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A32" s="1">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="B32" s="1" t="s">
-        <v>18</v>
+        <v>24</v>
       </c>
       <c r="C32" s="1" t="s">
         <v>6</v>
@@ -2564,10 +2566,10 @@
     </row>
     <row r="33" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A33" s="1">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="B33" s="1" t="s">
-        <v>23</v>
+        <v>17</v>
       </c>
       <c r="C33" s="1" t="s">
         <v>6</v>
@@ -2575,10 +2577,10 @@
     </row>
     <row r="34" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A34" s="1">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="B34" s="1" t="s">
-        <v>50</v>
+        <v>16</v>
       </c>
       <c r="C34" s="1" t="s">
         <v>6</v>
@@ -2586,10 +2588,10 @@
     </row>
     <row r="35" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A35" s="1">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="B35" s="1" t="s">
-        <v>51</v>
+        <v>21</v>
       </c>
       <c r="C35" s="1" t="s">
         <v>6</v>
@@ -2597,10 +2599,10 @@
     </row>
     <row r="36" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A36" s="1">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="B36" s="1" t="s">
-        <v>9</v>
+        <v>18</v>
       </c>
       <c r="C36" s="1" t="s">
         <v>6</v>
@@ -2608,12 +2610,56 @@
     </row>
     <row r="37" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A37" s="1">
+        <v>15</v>
+      </c>
+      <c r="B37" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="C37" s="1" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="38" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A38" s="1">
+        <v>16</v>
+      </c>
+      <c r="B38" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="C38" s="1" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="39" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A39" s="1">
+        <v>17</v>
+      </c>
+      <c r="B39" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="C39" s="1" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="40" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A40" s="1">
         <v>18</v>
       </c>
-      <c r="B37" s="1" t="s">
+      <c r="B40" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="C40" s="1" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="41" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A41" s="1">
+        <v>19</v>
+      </c>
+      <c r="B41" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="C37" s="1" t="s">
+      <c r="C41" s="1" t="s">
         <v>6</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Dash Bebras 2025 e 2024
</commit_message>
<xml_diff>
--- a/Bases/Navegacao_Menu.xlsx
+++ b/Bases/Navegacao_Menu.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\djdan\Documents\GitHub\Dash-Upmat\Bases\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8A41AA8E-60E6-4809-A56D-F5361B30E5A8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4816A14F-C5D6-46C5-9922-4A09F63E7DB5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="24240" windowHeight="13020" activeTab="1" xr2:uid="{F34CCB2F-E2D2-4F06-83D1-8921BB237BC6}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="392" uniqueCount="62">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="402" uniqueCount="63">
   <si>
     <t>Ordem</t>
   </si>
@@ -225,6 +225,9 @@
   </si>
   <si>
     <t>Experience 2026</t>
+  </si>
+  <si>
+    <t>Engajamento Experience 2026</t>
   </si>
 </sst>
 </file>
@@ -1270,7 +1273,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C7F7F84F-51F4-4AA7-8488-D6CFB2C033F7}">
-  <dimension ref="A1:C82"/>
+  <dimension ref="A1:C87"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="42.5703125" bestFit="1" customWidth="1"/>
@@ -1601,7 +1604,7 @@
         <v>8</v>
       </c>
       <c r="B30" s="1" t="s">
-        <v>36</v>
+        <v>30</v>
       </c>
       <c r="C30" s="1" t="s">
         <v>5</v>
@@ -1612,7 +1615,7 @@
         <v>8</v>
       </c>
       <c r="B31" s="1" t="s">
-        <v>36</v>
+        <v>30</v>
       </c>
       <c r="C31" s="1" t="s">
         <v>4</v>
@@ -1623,7 +1626,7 @@
         <v>8</v>
       </c>
       <c r="B32" s="1" t="s">
-        <v>36</v>
+        <v>30</v>
       </c>
       <c r="C32" s="1" t="s">
         <v>6</v>
@@ -1631,13 +1634,13 @@
     </row>
     <row r="33" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A33" s="1">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B33" s="1" t="s">
-        <v>36</v>
-      </c>
-      <c r="C33" t="s">
-        <v>49</v>
+        <v>28</v>
+      </c>
+      <c r="C33" s="1" t="s">
+        <v>5</v>
       </c>
     </row>
     <row r="34" spans="1:3" x14ac:dyDescent="0.25">
@@ -1645,10 +1648,10 @@
         <v>9</v>
       </c>
       <c r="B34" s="1" t="s">
-        <v>45</v>
+        <v>28</v>
       </c>
       <c r="C34" s="1" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="35" spans="1:3" x14ac:dyDescent="0.25">
@@ -1656,21 +1659,21 @@
         <v>9</v>
       </c>
       <c r="B35" s="1" t="s">
-        <v>45</v>
+        <v>28</v>
       </c>
       <c r="C35" s="1" t="s">
-        <v>4</v>
+        <v>6</v>
       </c>
     </row>
     <row r="36" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A36" s="1">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="B36" s="1" t="s">
         <v>45</v>
       </c>
       <c r="C36" s="1" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
     </row>
     <row r="37" spans="1:3" x14ac:dyDescent="0.25">
@@ -1678,7 +1681,7 @@
         <v>10</v>
       </c>
       <c r="B37" s="1" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="C37" s="1" t="s">
         <v>4</v>
@@ -1689,7 +1692,7 @@
         <v>10</v>
       </c>
       <c r="B38" s="1" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="C38" s="1" t="s">
         <v>6</v>
@@ -1697,13 +1700,13 @@
     </row>
     <row r="39" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A39" s="1">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B39" s="1" t="s">
         <v>46</v>
       </c>
       <c r="C39" s="1" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="40" spans="1:3" x14ac:dyDescent="0.25">
@@ -1711,10 +1714,10 @@
         <v>11</v>
       </c>
       <c r="B40" s="1" t="s">
-        <v>43</v>
+        <v>46</v>
       </c>
       <c r="C40" s="1" t="s">
-        <v>4</v>
+        <v>6</v>
       </c>
     </row>
     <row r="41" spans="1:3" x14ac:dyDescent="0.25">
@@ -1722,21 +1725,21 @@
         <v>11</v>
       </c>
       <c r="B41" s="1" t="s">
-        <v>43</v>
+        <v>46</v>
       </c>
       <c r="C41" s="1" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
     </row>
     <row r="42" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A42" s="1">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B42" s="1" t="s">
         <v>43</v>
       </c>
       <c r="C42" s="1" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="43" spans="1:3" x14ac:dyDescent="0.25">
@@ -1744,10 +1747,10 @@
         <v>12</v>
       </c>
       <c r="B43" s="1" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="C43" s="1" t="s">
-        <v>4</v>
+        <v>6</v>
       </c>
     </row>
     <row r="44" spans="1:3" x14ac:dyDescent="0.25">
@@ -1755,21 +1758,21 @@
         <v>12</v>
       </c>
       <c r="B44" s="1" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="C44" s="1" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
     </row>
     <row r="45" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A45" s="1">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B45" s="1" t="s">
         <v>44</v>
       </c>
       <c r="C45" s="1" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="46" spans="1:3" x14ac:dyDescent="0.25">
@@ -1777,21 +1780,21 @@
         <v>13</v>
       </c>
       <c r="B46" s="1" t="s">
-        <v>61</v>
+        <v>44</v>
       </c>
       <c r="C46" s="1" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="47" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A47" s="1">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B47" s="1" t="s">
-        <v>47</v>
+        <v>44</v>
       </c>
       <c r="C47" s="1" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
     </row>
     <row r="48" spans="1:3" x14ac:dyDescent="0.25">
@@ -1799,10 +1802,10 @@
         <v>14</v>
       </c>
       <c r="B48" s="1" t="s">
-        <v>47</v>
+        <v>61</v>
       </c>
       <c r="C48" s="1" t="s">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="49" spans="1:3" x14ac:dyDescent="0.25">
@@ -1810,21 +1813,21 @@
         <v>14</v>
       </c>
       <c r="B49" s="1" t="s">
-        <v>47</v>
+        <v>61</v>
       </c>
       <c r="C49" s="1" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="50" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A50" s="1">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B50" s="1" t="s">
-        <v>48</v>
+        <v>61</v>
       </c>
       <c r="C50" s="1" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
     </row>
     <row r="51" spans="1:3" x14ac:dyDescent="0.25">
@@ -1832,10 +1835,10 @@
         <v>15</v>
       </c>
       <c r="B51" s="1" t="s">
-        <v>48</v>
+        <v>62</v>
       </c>
       <c r="C51" s="1" t="s">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="52" spans="1:3" x14ac:dyDescent="0.25">
@@ -1843,21 +1846,21 @@
         <v>15</v>
       </c>
       <c r="B52" s="1" t="s">
-        <v>48</v>
+        <v>62</v>
       </c>
       <c r="C52" s="1" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="53" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A53" s="1">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B53" s="1" t="s">
-        <v>3</v>
+        <v>62</v>
       </c>
       <c r="C53" s="1" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
     </row>
     <row r="54" spans="1:3" x14ac:dyDescent="0.25">
@@ -1865,10 +1868,10 @@
         <v>16</v>
       </c>
       <c r="B54" s="1" t="s">
-        <v>3</v>
+        <v>36</v>
       </c>
       <c r="C54" s="1" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="55" spans="1:3" x14ac:dyDescent="0.25">
@@ -1876,32 +1879,32 @@
         <v>16</v>
       </c>
       <c r="B55" s="1" t="s">
-        <v>3</v>
+        <v>36</v>
       </c>
       <c r="C55" s="1" t="s">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="56" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A56" s="1">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B56" s="1" t="s">
-        <v>7</v>
+        <v>36</v>
       </c>
       <c r="C56" s="1" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
     </row>
     <row r="57" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A57" s="1">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B57" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="C57" s="1" t="s">
-        <v>5</v>
+        <v>36</v>
+      </c>
+      <c r="C57" t="s">
+        <v>49</v>
       </c>
     </row>
     <row r="58" spans="1:3" x14ac:dyDescent="0.25">
@@ -1909,29 +1912,29 @@
         <v>17</v>
       </c>
       <c r="B58" s="1" t="s">
-        <v>7</v>
+        <v>47</v>
       </c>
       <c r="C58" s="1" t="s">
-        <v>4</v>
+        <v>6</v>
       </c>
     </row>
     <row r="59" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A59" s="1">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="B59" s="1" t="s">
-        <v>41</v>
+        <v>47</v>
       </c>
       <c r="C59" s="1" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
     </row>
     <row r="60" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A60" s="1">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="B60" s="1" t="s">
-        <v>41</v>
+        <v>47</v>
       </c>
       <c r="C60" s="1" t="s">
         <v>5</v>
@@ -1942,29 +1945,29 @@
         <v>18</v>
       </c>
       <c r="B61" s="1" t="s">
-        <v>41</v>
+        <v>48</v>
       </c>
       <c r="C61" s="1" t="s">
-        <v>4</v>
+        <v>6</v>
       </c>
     </row>
     <row r="62" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A62" s="1">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="B62" s="1" t="s">
-        <v>35</v>
+        <v>48</v>
       </c>
       <c r="C62" s="1" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
     </row>
     <row r="63" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A63" s="1">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="B63" s="1" t="s">
-        <v>35</v>
+        <v>48</v>
       </c>
       <c r="C63" s="1" t="s">
         <v>5</v>
@@ -1975,32 +1978,32 @@
         <v>19</v>
       </c>
       <c r="B64" s="1" t="s">
-        <v>35</v>
+        <v>3</v>
       </c>
       <c r="C64" s="1" t="s">
-        <v>4</v>
+        <v>6</v>
       </c>
     </row>
     <row r="65" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A65" s="1">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B65" s="1" t="s">
-        <v>34</v>
+        <v>3</v>
       </c>
       <c r="C65" s="1" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
     </row>
     <row r="66" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A66" s="1">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B66" s="1" t="s">
-        <v>34</v>
+        <v>3</v>
       </c>
       <c r="C66" s="1" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="67" spans="1:3" x14ac:dyDescent="0.25">
@@ -2008,40 +2011,40 @@
         <v>20</v>
       </c>
       <c r="B67" s="1" t="s">
-        <v>34</v>
+        <v>7</v>
       </c>
       <c r="C67" s="1" t="s">
-        <v>4</v>
+        <v>6</v>
       </c>
     </row>
     <row r="68" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A68" s="1">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B68" s="1" t="s">
-        <v>33</v>
+        <v>7</v>
       </c>
       <c r="C68" s="1" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
     </row>
     <row r="69" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A69" s="1">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B69" s="1" t="s">
-        <v>33</v>
+        <v>7</v>
       </c>
       <c r="C69" s="1" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="70" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A70" s="1">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="B70" s="1" t="s">
-        <v>32</v>
+        <v>41</v>
       </c>
       <c r="C70" s="1" t="s">
         <v>6</v>
@@ -2049,10 +2052,10 @@
     </row>
     <row r="71" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A71" s="1">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="B71" s="1" t="s">
-        <v>32</v>
+        <v>41</v>
       </c>
       <c r="C71" s="1" t="s">
         <v>5</v>
@@ -2060,65 +2063,65 @@
     </row>
     <row r="72" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A72" s="1">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="B72" s="1" t="s">
-        <v>31</v>
+        <v>41</v>
       </c>
       <c r="C72" s="1" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
     </row>
     <row r="73" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A73" s="1">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="B73" s="1" t="s">
-        <v>31</v>
+        <v>35</v>
       </c>
       <c r="C73" s="1" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="74" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A74" s="1">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="B74" s="1" t="s">
-        <v>30</v>
+        <v>35</v>
       </c>
       <c r="C74" s="1" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
     </row>
     <row r="75" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A75" s="1">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="B75" s="1" t="s">
-        <v>30</v>
+        <v>35</v>
       </c>
       <c r="C75" s="1" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
     </row>
     <row r="76" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A76" s="1">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="B76" s="1" t="s">
-        <v>30</v>
+        <v>34</v>
       </c>
       <c r="C76" s="1" t="s">
-        <v>4</v>
+        <v>6</v>
       </c>
     </row>
     <row r="77" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A77" s="1">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="B77" s="1" t="s">
-        <v>28</v>
+        <v>34</v>
       </c>
       <c r="C77" s="1" t="s">
         <v>5</v>
@@ -2126,32 +2129,32 @@
     </row>
     <row r="78" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A78" s="1">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="B78" s="1" t="s">
-        <v>28</v>
+        <v>34</v>
       </c>
       <c r="C78" s="1" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
     </row>
     <row r="79" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A79" s="1">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="B79" s="1" t="s">
-        <v>28</v>
+        <v>33</v>
       </c>
       <c r="C79" s="1" t="s">
-        <v>4</v>
+        <v>6</v>
       </c>
     </row>
     <row r="80" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A80" s="1">
-        <v>26</v>
-      </c>
-      <c r="B80" t="s">
-        <v>29</v>
+        <v>24</v>
+      </c>
+      <c r="B80" s="1" t="s">
+        <v>33</v>
       </c>
       <c r="C80" s="1" t="s">
         <v>5</v>
@@ -2159,10 +2162,10 @@
     </row>
     <row r="81" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A81" s="1">
-        <v>26</v>
-      </c>
-      <c r="B81" t="s">
-        <v>29</v>
+        <v>25</v>
+      </c>
+      <c r="B81" s="1" t="s">
+        <v>32</v>
       </c>
       <c r="C81" s="1" t="s">
         <v>6</v>
@@ -2170,12 +2173,67 @@
     </row>
     <row r="82" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A82" s="1">
+        <v>25</v>
+      </c>
+      <c r="B82" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="C82" s="1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="83" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A83" s="1">
         <v>26</v>
       </c>
-      <c r="B82" t="s">
+      <c r="B83" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="C83" s="1" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="84" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A84" s="1">
+        <v>26</v>
+      </c>
+      <c r="B84" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="C84" s="1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="85" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A85" s="1">
+        <v>27</v>
+      </c>
+      <c r="B85" t="s">
         <v>29</v>
       </c>
-      <c r="C82" s="1" t="s">
+      <c r="C85" s="1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="86" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A86" s="1">
+        <v>27</v>
+      </c>
+      <c r="B86" t="s">
+        <v>29</v>
+      </c>
+      <c r="C86" s="1" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="87" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A87" s="1">
+        <v>27</v>
+      </c>
+      <c r="B87" t="s">
+        <v>29</v>
+      </c>
+      <c r="C87" s="1" t="s">
         <v>4</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Melhoras Arquitetura Canguru e Bebras
</commit_message>
<xml_diff>
--- a/Bases/Navegacao_Menu.xlsx
+++ b/Bases/Navegacao_Menu.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\djdan\Documents\GitHub\Dash-Upmat\Bases\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{93E9933E-9F7D-4D71-8044-ECB802058851}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CF283FB0-36AD-4B60-BE88-A435C25C2B28}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="24240" windowHeight="13020" activeTab="4" xr2:uid="{F34CCB2F-E2D2-4F06-83D1-8921BB237BC6}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="24240" windowHeight="13020" activeTab="5" xr2:uid="{F34CCB2F-E2D2-4F06-83D1-8921BB237BC6}"/>
   </bookViews>
   <sheets>
     <sheet name="Olitef 2025" sheetId="2" r:id="rId1"/>
@@ -44,7 +44,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="739" uniqueCount="88">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="855" uniqueCount="111">
   <si>
     <t>Ordem</t>
   </si>
@@ -154,9 +154,6 @@
     <t>Potencial de Conversão Inscrições 2025 - Part1</t>
   </si>
   <si>
-    <t>Migração Experience 2025 x 2026</t>
-  </si>
-  <si>
     <t>Migração de Plano 2025 x 2026</t>
   </si>
   <si>
@@ -229,12 +226,6 @@
     <t>Potencial de Conversão 2024 - Part2</t>
   </si>
   <si>
-    <t>Experience 2026</t>
-  </si>
-  <si>
-    <t>Engajamento Experience 2026</t>
-  </si>
-  <si>
     <t>Pedido de Medalhas 2025</t>
   </si>
   <si>
@@ -308,6 +299,84 @@
   </si>
   <si>
     <t>Migração Canguru Experience 2025 x 2026</t>
+  </si>
+  <si>
+    <t>1a</t>
+  </si>
+  <si>
+    <t>1b</t>
+  </si>
+  <si>
+    <t>1c</t>
+  </si>
+  <si>
+    <t>1d</t>
+  </si>
+  <si>
+    <t>1e</t>
+  </si>
+  <si>
+    <t>1f</t>
+  </si>
+  <si>
+    <t>1g</t>
+  </si>
+  <si>
+    <t>1h</t>
+  </si>
+  <si>
+    <t>1i</t>
+  </si>
+  <si>
+    <t>1j</t>
+  </si>
+  <si>
+    <t>1k</t>
+  </si>
+  <si>
+    <t>1l</t>
+  </si>
+  <si>
+    <t>1m</t>
+  </si>
+  <si>
+    <t>1n</t>
+  </si>
+  <si>
+    <t>1o</t>
+  </si>
+  <si>
+    <t>1p</t>
+  </si>
+  <si>
+    <t>1q</t>
+  </si>
+  <si>
+    <t>1r</t>
+  </si>
+  <si>
+    <t>1s</t>
+  </si>
+  <si>
+    <t>1t</t>
+  </si>
+  <si>
+    <t>1u</t>
+  </si>
+  <si>
+    <t>1v</t>
+  </si>
+  <si>
+    <t>1w</t>
+  </si>
+  <si>
+    <t>1y</t>
+  </si>
+  <si>
+    <t>1z</t>
+  </si>
+  <si>
+    <t>1x</t>
   </si>
 </sst>
 </file>
@@ -1361,7 +1430,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C7F7F84F-51F4-4AA7-8488-D6CFB2C033F7}">
-  <dimension ref="A1:C87"/>
+  <dimension ref="A1:C74"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="42.5703125" bestFit="1" customWidth="1"/>
@@ -1420,7 +1489,7 @@
         <v>25</v>
       </c>
       <c r="C5" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
@@ -1464,7 +1533,7 @@
         <v>26</v>
       </c>
       <c r="C9" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.25">
@@ -1472,7 +1541,7 @@
         <v>3</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C10" s="1" t="s">
         <v>4</v>
@@ -1483,7 +1552,7 @@
         <v>3</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C11" s="1" t="s">
         <v>6</v>
@@ -1494,7 +1563,7 @@
         <v>3</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C12" s="1" t="s">
         <v>5</v>
@@ -1505,10 +1574,10 @@
         <v>3</v>
       </c>
       <c r="B13" s="1" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C13" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.25">
@@ -1516,7 +1585,7 @@
         <v>4</v>
       </c>
       <c r="B14" s="1" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="C14" s="1" t="s">
         <v>4</v>
@@ -1527,7 +1596,7 @@
         <v>4</v>
       </c>
       <c r="B15" s="1" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="C15" s="1" t="s">
         <v>6</v>
@@ -1538,7 +1607,7 @@
         <v>4</v>
       </c>
       <c r="B16" s="1" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="C16" s="1" t="s">
         <v>5</v>
@@ -1549,10 +1618,10 @@
         <v>4</v>
       </c>
       <c r="B17" s="1" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="C17" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.25">
@@ -1560,7 +1629,7 @@
         <v>5</v>
       </c>
       <c r="B18" s="1" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="C18" s="1" t="s">
         <v>4</v>
@@ -1571,7 +1640,7 @@
         <v>5</v>
       </c>
       <c r="B19" s="1" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="C19" s="1" t="s">
         <v>5</v>
@@ -1582,7 +1651,7 @@
         <v>5</v>
       </c>
       <c r="B20" s="1" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="C20" s="1" t="s">
         <v>6</v>
@@ -1593,10 +1662,10 @@
         <v>5</v>
       </c>
       <c r="B21" s="1" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="C21" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
     </row>
     <row r="22" spans="1:3" x14ac:dyDescent="0.25">
@@ -1604,7 +1673,7 @@
         <v>6</v>
       </c>
       <c r="B22" s="1" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="C22" s="1" t="s">
         <v>4</v>
@@ -1615,7 +1684,7 @@
         <v>6</v>
       </c>
       <c r="B23" s="1" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="C23" s="1" t="s">
         <v>5</v>
@@ -1626,7 +1695,7 @@
         <v>6</v>
       </c>
       <c r="B24" s="1" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="C24" s="1" t="s">
         <v>6</v>
@@ -1637,10 +1706,10 @@
         <v>6</v>
       </c>
       <c r="B25" s="1" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="C25" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
     </row>
     <row r="26" spans="1:3" x14ac:dyDescent="0.25">
@@ -1648,7 +1717,7 @@
         <v>7</v>
       </c>
       <c r="B26" s="1" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="C26" s="1" t="s">
         <v>6</v>
@@ -1659,7 +1728,7 @@
         <v>7</v>
       </c>
       <c r="B27" s="1" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="C27" s="1" t="s">
         <v>5</v>
@@ -1670,7 +1739,7 @@
         <v>7</v>
       </c>
       <c r="B28" s="1" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="C28" s="1" t="s">
         <v>4</v>
@@ -1681,10 +1750,10 @@
         <v>7</v>
       </c>
       <c r="B29" s="1" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="C29" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
     </row>
     <row r="30" spans="1:3" x14ac:dyDescent="0.25">
@@ -1758,7 +1827,7 @@
         <v>10</v>
       </c>
       <c r="B36" s="1" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="C36" s="1" t="s">
         <v>5</v>
@@ -1769,7 +1838,7 @@
         <v>10</v>
       </c>
       <c r="B37" s="1" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="C37" s="1" t="s">
         <v>4</v>
@@ -1780,7 +1849,7 @@
         <v>10</v>
       </c>
       <c r="B38" s="1" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="C38" s="1" t="s">
         <v>6</v>
@@ -1791,7 +1860,7 @@
         <v>11</v>
       </c>
       <c r="B39" s="1" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="C39" s="1" t="s">
         <v>4</v>
@@ -1802,7 +1871,7 @@
         <v>11</v>
       </c>
       <c r="B40" s="1" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="C40" s="1" t="s">
         <v>6</v>
@@ -1813,7 +1882,7 @@
         <v>11</v>
       </c>
       <c r="B41" s="1" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="C41" s="1" t="s">
         <v>5</v>
@@ -1824,7 +1893,7 @@
         <v>12</v>
       </c>
       <c r="B42" s="1" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="C42" s="1" t="s">
         <v>4</v>
@@ -1835,7 +1904,7 @@
         <v>12</v>
       </c>
       <c r="B43" s="1" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="C43" s="1" t="s">
         <v>6</v>
@@ -1846,7 +1915,7 @@
         <v>12</v>
       </c>
       <c r="B44" s="1" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="C44" s="1" t="s">
         <v>5</v>
@@ -1857,7 +1926,7 @@
         <v>13</v>
       </c>
       <c r="B45" s="1" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="C45" s="1" t="s">
         <v>4</v>
@@ -1868,7 +1937,7 @@
         <v>13</v>
       </c>
       <c r="B46" s="1" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="C46" s="1" t="s">
         <v>6</v>
@@ -1879,7 +1948,7 @@
         <v>13</v>
       </c>
       <c r="B47" s="1" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="C47" s="1" t="s">
         <v>5</v>
@@ -1890,10 +1959,10 @@
         <v>14</v>
       </c>
       <c r="B48" s="1" t="s">
-        <v>61</v>
+        <v>46</v>
       </c>
       <c r="C48" s="1" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="49" spans="1:3" x14ac:dyDescent="0.25">
@@ -1901,10 +1970,10 @@
         <v>14</v>
       </c>
       <c r="B49" s="1" t="s">
-        <v>61</v>
+        <v>46</v>
       </c>
       <c r="C49" s="1" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
     </row>
     <row r="50" spans="1:3" x14ac:dyDescent="0.25">
@@ -1912,10 +1981,10 @@
         <v>14</v>
       </c>
       <c r="B50" s="1" t="s">
-        <v>61</v>
+        <v>46</v>
       </c>
       <c r="C50" s="1" t="s">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="51" spans="1:3" x14ac:dyDescent="0.25">
@@ -1923,10 +1992,10 @@
         <v>15</v>
       </c>
       <c r="B51" s="1" t="s">
-        <v>62</v>
+        <v>3</v>
       </c>
       <c r="C51" s="1" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="52" spans="1:3" x14ac:dyDescent="0.25">
@@ -1934,10 +2003,10 @@
         <v>15</v>
       </c>
       <c r="B52" s="1" t="s">
-        <v>62</v>
+        <v>3</v>
       </c>
       <c r="C52" s="1" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
     </row>
     <row r="53" spans="1:3" x14ac:dyDescent="0.25">
@@ -1945,7 +2014,7 @@
         <v>15</v>
       </c>
       <c r="B53" s="1" t="s">
-        <v>62</v>
+        <v>3</v>
       </c>
       <c r="C53" s="1" t="s">
         <v>4</v>
@@ -1956,7 +2025,7 @@
         <v>16</v>
       </c>
       <c r="B54" s="1" t="s">
-        <v>36</v>
+        <v>7</v>
       </c>
       <c r="C54" s="1" t="s">
         <v>6</v>
@@ -1967,7 +2036,7 @@
         <v>16</v>
       </c>
       <c r="B55" s="1" t="s">
-        <v>36</v>
+        <v>7</v>
       </c>
       <c r="C55" s="1" t="s">
         <v>5</v>
@@ -1978,7 +2047,7 @@
         <v>16</v>
       </c>
       <c r="B56" s="1" t="s">
-        <v>36</v>
+        <v>7</v>
       </c>
       <c r="C56" s="1" t="s">
         <v>4</v>
@@ -1986,13 +2055,13 @@
     </row>
     <row r="57" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A57" s="1">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="B57" s="1" t="s">
-        <v>36</v>
-      </c>
-      <c r="C57" t="s">
-        <v>49</v>
+        <v>40</v>
+      </c>
+      <c r="C57" s="1" t="s">
+        <v>6</v>
       </c>
     </row>
     <row r="58" spans="1:3" x14ac:dyDescent="0.25">
@@ -2000,10 +2069,10 @@
         <v>17</v>
       </c>
       <c r="B58" s="1" t="s">
-        <v>47</v>
+        <v>40</v>
       </c>
       <c r="C58" s="1" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
     </row>
     <row r="59" spans="1:3" x14ac:dyDescent="0.25">
@@ -2011,7 +2080,7 @@
         <v>17</v>
       </c>
       <c r="B59" s="1" t="s">
-        <v>47</v>
+        <v>40</v>
       </c>
       <c r="C59" s="1" t="s">
         <v>4</v>
@@ -2019,13 +2088,13 @@
     </row>
     <row r="60" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A60" s="1">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="B60" s="1" t="s">
-        <v>47</v>
+        <v>35</v>
       </c>
       <c r="C60" s="1" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="61" spans="1:3" x14ac:dyDescent="0.25">
@@ -2033,10 +2102,10 @@
         <v>18</v>
       </c>
       <c r="B61" s="1" t="s">
-        <v>48</v>
+        <v>35</v>
       </c>
       <c r="C61" s="1" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
     </row>
     <row r="62" spans="1:3" x14ac:dyDescent="0.25">
@@ -2044,7 +2113,7 @@
         <v>18</v>
       </c>
       <c r="B62" s="1" t="s">
-        <v>48</v>
+        <v>35</v>
       </c>
       <c r="C62" s="1" t="s">
         <v>4</v>
@@ -2052,13 +2121,13 @@
     </row>
     <row r="63" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A63" s="1">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="B63" s="1" t="s">
-        <v>48</v>
+        <v>34</v>
       </c>
       <c r="C63" s="1" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="64" spans="1:3" x14ac:dyDescent="0.25">
@@ -2066,10 +2135,10 @@
         <v>19</v>
       </c>
       <c r="B64" s="1" t="s">
-        <v>3</v>
+        <v>34</v>
       </c>
       <c r="C64" s="1" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
     </row>
     <row r="65" spans="1:3" x14ac:dyDescent="0.25">
@@ -2077,21 +2146,21 @@
         <v>19</v>
       </c>
       <c r="B65" s="1" t="s">
-        <v>3</v>
+        <v>34</v>
       </c>
       <c r="C65" s="1" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="66" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A66" s="1">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="B66" s="1" t="s">
-        <v>3</v>
+        <v>33</v>
       </c>
       <c r="C66" s="1" t="s">
-        <v>4</v>
+        <v>6</v>
       </c>
     </row>
     <row r="67" spans="1:3" x14ac:dyDescent="0.25">
@@ -2099,40 +2168,40 @@
         <v>20</v>
       </c>
       <c r="B67" s="1" t="s">
-        <v>7</v>
+        <v>33</v>
       </c>
       <c r="C67" s="1" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
     </row>
     <row r="68" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A68" s="1">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="B68" s="1" t="s">
-        <v>7</v>
+        <v>32</v>
       </c>
       <c r="C68" s="1" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="69" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A69" s="1">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="B69" s="1" t="s">
-        <v>7</v>
+        <v>32</v>
       </c>
       <c r="C69" s="1" t="s">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="70" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A70" s="1">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="B70" s="1" t="s">
-        <v>41</v>
+        <v>31</v>
       </c>
       <c r="C70" s="1" t="s">
         <v>6</v>
@@ -2140,10 +2209,10 @@
     </row>
     <row r="71" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A71" s="1">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="B71" s="1" t="s">
-        <v>41</v>
+        <v>31</v>
       </c>
       <c r="C71" s="1" t="s">
         <v>5</v>
@@ -2151,21 +2220,21 @@
     </row>
     <row r="72" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A72" s="1">
-        <v>21</v>
-      </c>
-      <c r="B72" s="1" t="s">
-        <v>41</v>
+        <v>23</v>
+      </c>
+      <c r="B72" t="s">
+        <v>29</v>
       </c>
       <c r="C72" s="1" t="s">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="73" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A73" s="1">
-        <v>22</v>
-      </c>
-      <c r="B73" s="1" t="s">
-        <v>35</v>
+        <v>23</v>
+      </c>
+      <c r="B73" t="s">
+        <v>29</v>
       </c>
       <c r="C73" s="1" t="s">
         <v>6</v>
@@ -2173,155 +2242,12 @@
     </row>
     <row r="74" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A74" s="1">
-        <v>22</v>
-      </c>
-      <c r="B74" s="1" t="s">
-        <v>35</v>
+        <v>23</v>
+      </c>
+      <c r="B74" t="s">
+        <v>29</v>
       </c>
       <c r="C74" s="1" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="75" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A75" s="1">
-        <v>22</v>
-      </c>
-      <c r="B75" s="1" t="s">
-        <v>35</v>
-      </c>
-      <c r="C75" s="1" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="76" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A76" s="1">
-        <v>23</v>
-      </c>
-      <c r="B76" s="1" t="s">
-        <v>34</v>
-      </c>
-      <c r="C76" s="1" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="77" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A77" s="1">
-        <v>23</v>
-      </c>
-      <c r="B77" s="1" t="s">
-        <v>34</v>
-      </c>
-      <c r="C77" s="1" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="78" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A78" s="1">
-        <v>23</v>
-      </c>
-      <c r="B78" s="1" t="s">
-        <v>34</v>
-      </c>
-      <c r="C78" s="1" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="79" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A79" s="1">
-        <v>24</v>
-      </c>
-      <c r="B79" s="1" t="s">
-        <v>33</v>
-      </c>
-      <c r="C79" s="1" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="80" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A80" s="1">
-        <v>24</v>
-      </c>
-      <c r="B80" s="1" t="s">
-        <v>33</v>
-      </c>
-      <c r="C80" s="1" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="81" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A81" s="1">
-        <v>25</v>
-      </c>
-      <c r="B81" s="1" t="s">
-        <v>32</v>
-      </c>
-      <c r="C81" s="1" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="82" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A82" s="1">
-        <v>25</v>
-      </c>
-      <c r="B82" s="1" t="s">
-        <v>32</v>
-      </c>
-      <c r="C82" s="1" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="83" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A83" s="1">
-        <v>26</v>
-      </c>
-      <c r="B83" s="1" t="s">
-        <v>31</v>
-      </c>
-      <c r="C83" s="1" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="84" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A84" s="1">
-        <v>26</v>
-      </c>
-      <c r="B84" s="1" t="s">
-        <v>31</v>
-      </c>
-      <c r="C84" s="1" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="85" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A85" s="1">
-        <v>27</v>
-      </c>
-      <c r="B85" t="s">
-        <v>29</v>
-      </c>
-      <c r="C85" s="1" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="86" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A86" s="1">
-        <v>27</v>
-      </c>
-      <c r="B86" t="s">
-        <v>29</v>
-      </c>
-      <c r="C86" s="1" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="87" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A87" s="1">
-        <v>27</v>
-      </c>
-      <c r="B87" t="s">
-        <v>29</v>
-      </c>
-      <c r="C87" s="1" t="s">
         <v>4</v>
       </c>
     </row>
@@ -2497,7 +2423,7 @@
         <v>3</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>74</v>
+        <v>71</v>
       </c>
       <c r="C10" s="1" t="s">
         <v>4</v>
@@ -2508,7 +2434,7 @@
         <v>3</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>74</v>
+        <v>71</v>
       </c>
       <c r="C11" s="1" t="s">
         <v>6</v>
@@ -2519,7 +2445,7 @@
         <v>3</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>74</v>
+        <v>71</v>
       </c>
       <c r="C12" s="1" t="s">
         <v>5</v>
@@ -2530,7 +2456,7 @@
         <v>4</v>
       </c>
       <c r="B13" s="1" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="C13" s="1" t="s">
         <v>19</v>
@@ -2541,7 +2467,7 @@
         <v>4</v>
       </c>
       <c r="B14" s="1" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="C14" s="1" t="s">
         <v>6</v>
@@ -2552,7 +2478,7 @@
         <v>5</v>
       </c>
       <c r="B15" s="1" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C15" s="1" t="s">
         <v>6</v>
@@ -2563,7 +2489,7 @@
         <v>5</v>
       </c>
       <c r="B16" s="1" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C16" s="1" t="s">
         <v>4</v>
@@ -2574,7 +2500,7 @@
         <v>5</v>
       </c>
       <c r="B17" s="1" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C17" s="1" t="s">
         <v>5</v>
@@ -2585,7 +2511,7 @@
         <v>6</v>
       </c>
       <c r="B18" s="1" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="C18" s="1" t="s">
         <v>19</v>
@@ -2596,7 +2522,7 @@
         <v>6</v>
       </c>
       <c r="B19" s="1" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="C19" s="1" t="s">
         <v>4</v>
@@ -2607,7 +2533,7 @@
         <v>6</v>
       </c>
       <c r="B20" s="1" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="C20" s="1" t="s">
         <v>5</v>
@@ -2618,7 +2544,7 @@
         <v>6</v>
       </c>
       <c r="B21" s="1" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="C21" s="1" t="s">
         <v>6</v>
@@ -2794,7 +2720,7 @@
         <v>13</v>
       </c>
       <c r="B37" s="1" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="C37" s="1" t="s">
         <v>6</v>
@@ -2816,7 +2742,7 @@
         <v>15</v>
       </c>
       <c r="B39" s="1" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="C39" s="1" t="s">
         <v>19</v>
@@ -2827,7 +2753,7 @@
         <v>15</v>
       </c>
       <c r="B40" s="1" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="C40" s="1" t="s">
         <v>4</v>
@@ -2838,7 +2764,7 @@
         <v>15</v>
       </c>
       <c r="B41" s="1" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="C41" s="1" t="s">
         <v>5</v>
@@ -2849,7 +2775,7 @@
         <v>15</v>
       </c>
       <c r="B42" s="1" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="C42" s="1" t="s">
         <v>6</v>
@@ -2860,7 +2786,7 @@
         <v>16</v>
       </c>
       <c r="B43" s="1" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="C43" s="1" t="s">
         <v>19</v>
@@ -2871,7 +2797,7 @@
         <v>16</v>
       </c>
       <c r="B44" s="1" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="C44" s="1" t="s">
         <v>4</v>
@@ -2882,7 +2808,7 @@
         <v>16</v>
       </c>
       <c r="B45" s="1" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="C45" s="1" t="s">
         <v>5</v>
@@ -2893,7 +2819,7 @@
         <v>16</v>
       </c>
       <c r="B46" s="1" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="C46" s="1" t="s">
         <v>6</v>
@@ -2904,7 +2830,7 @@
         <v>17</v>
       </c>
       <c r="B47" s="1" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="C47" s="1" t="s">
         <v>6</v>
@@ -2915,7 +2841,7 @@
         <v>18</v>
       </c>
       <c r="B48" s="1" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="C48" s="1" t="s">
         <v>6</v>
@@ -2926,7 +2852,7 @@
         <v>19</v>
       </c>
       <c r="B49" s="1" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="C49" s="1" t="s">
         <v>6</v>
@@ -2948,7 +2874,7 @@
         <v>21</v>
       </c>
       <c r="B51" s="1" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="C51" s="1" t="s">
         <v>6</v>
@@ -2959,7 +2885,7 @@
         <v>22</v>
       </c>
       <c r="B52" s="1" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="C52" s="1" t="s">
         <v>6</v>
@@ -2970,7 +2896,7 @@
         <v>23</v>
       </c>
       <c r="B53" s="1" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="C53" s="1" t="s">
         <v>6</v>
@@ -3007,7 +2933,7 @@
         <v>1</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>84</v>
+        <v>81</v>
       </c>
       <c r="C2" s="1" t="s">
         <v>5</v>
@@ -3018,7 +2944,7 @@
         <v>1</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>84</v>
+        <v>81</v>
       </c>
       <c r="C3" s="1" t="s">
         <v>6</v>
@@ -3029,7 +2955,7 @@
         <v>1</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>84</v>
+        <v>81</v>
       </c>
       <c r="C4" s="1" t="s">
         <v>4</v>
@@ -3040,10 +2966,10 @@
         <v>1</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>84</v>
+        <v>81</v>
       </c>
       <c r="C5" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
@@ -3051,7 +2977,7 @@
         <v>2</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>85</v>
+        <v>82</v>
       </c>
       <c r="C6" s="1" t="s">
         <v>5</v>
@@ -3062,7 +2988,7 @@
         <v>2</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>85</v>
+        <v>82</v>
       </c>
       <c r="C7" s="1" t="s">
         <v>6</v>
@@ -3073,7 +2999,7 @@
         <v>2</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>85</v>
+        <v>82</v>
       </c>
       <c r="C8" s="1" t="s">
         <v>4</v>
@@ -3084,10 +3010,10 @@
         <v>2</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>85</v>
+        <v>82</v>
       </c>
       <c r="C9" s="3" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.25">
@@ -3095,7 +3021,7 @@
         <v>3</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>86</v>
+        <v>83</v>
       </c>
       <c r="C10" s="1" t="s">
         <v>5</v>
@@ -3106,7 +3032,7 @@
         <v>3</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>86</v>
+        <v>83</v>
       </c>
       <c r="C11" s="1" t="s">
         <v>6</v>
@@ -3117,7 +3043,7 @@
         <v>3</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>86</v>
+        <v>83</v>
       </c>
       <c r="C12" s="1" t="s">
         <v>4</v>
@@ -3128,10 +3054,10 @@
         <v>3</v>
       </c>
       <c r="B13" s="1" t="s">
-        <v>86</v>
+        <v>83</v>
       </c>
       <c r="C13" s="3" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.25">
@@ -3139,7 +3065,7 @@
         <v>4</v>
       </c>
       <c r="B14" s="1" t="s">
-        <v>87</v>
+        <v>84</v>
       </c>
       <c r="C14" s="1" t="s">
         <v>6</v>
@@ -3150,7 +3076,7 @@
         <v>4</v>
       </c>
       <c r="B15" s="1" t="s">
-        <v>87</v>
+        <v>84</v>
       </c>
       <c r="C15" s="1" t="s">
         <v>5</v>
@@ -3161,7 +3087,7 @@
         <v>4</v>
       </c>
       <c r="B16" s="1" t="s">
-        <v>87</v>
+        <v>84</v>
       </c>
       <c r="C16" s="1" t="s">
         <v>4</v>
@@ -3172,10 +3098,10 @@
         <v>4</v>
       </c>
       <c r="B17" s="1" t="s">
-        <v>87</v>
+        <v>84</v>
       </c>
       <c r="C17" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.25">
@@ -3183,7 +3109,7 @@
         <v>5</v>
       </c>
       <c r="B18" s="1" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="C18" s="1" t="s">
         <v>6</v>
@@ -3194,7 +3120,7 @@
         <v>5</v>
       </c>
       <c r="B19" s="1" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="C19" s="1" t="s">
         <v>4</v>
@@ -3205,7 +3131,7 @@
         <v>5</v>
       </c>
       <c r="B20" s="1" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="C20" s="1" t="s">
         <v>5</v>
@@ -3216,10 +3142,10 @@
         <v>5</v>
       </c>
       <c r="B21" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="C21" t="s">
         <v>48</v>
-      </c>
-      <c r="C21" t="s">
-        <v>49</v>
       </c>
     </row>
   </sheetData>
@@ -3229,7 +3155,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5AD31D2E-82F9-4A53-8E31-D57E1126423D}">
-  <dimension ref="A1:F73"/>
+  <dimension ref="A1:F86"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="42.5703125" bestFit="1" customWidth="1"/>
@@ -3249,18 +3175,18 @@
         <v>2</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>75</v>
+        <v>72</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>76</v>
+        <v>73</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>77</v>
+        <v>74</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A2" s="1">
-        <v>1</v>
+      <c r="A2" s="1" t="s">
+        <v>85</v>
       </c>
       <c r="B2" s="1" t="s">
         <v>25</v>
@@ -3269,18 +3195,18 @@
         <v>4</v>
       </c>
       <c r="D2" t="s">
-        <v>78</v>
+        <v>75</v>
       </c>
       <c r="E2">
         <v>1</v>
       </c>
       <c r="F2" t="s">
-        <v>81</v>
+        <v>78</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A3" s="1">
-        <v>1</v>
+      <c r="A3" s="1" t="s">
+        <v>85</v>
       </c>
       <c r="B3" s="1" t="s">
         <v>25</v>
@@ -3289,18 +3215,18 @@
         <v>5</v>
       </c>
       <c r="D3" t="s">
-        <v>78</v>
+        <v>75</v>
       </c>
       <c r="E3">
         <v>1</v>
       </c>
       <c r="F3" t="s">
-        <v>81</v>
+        <v>78</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A4" s="1">
-        <v>1</v>
+      <c r="A4" s="1" t="s">
+        <v>85</v>
       </c>
       <c r="B4" s="1" t="s">
         <v>25</v>
@@ -3309,38 +3235,38 @@
         <v>6</v>
       </c>
       <c r="D4" t="s">
-        <v>78</v>
+        <v>75</v>
       </c>
       <c r="E4">
         <v>1</v>
       </c>
       <c r="F4" t="s">
-        <v>81</v>
+        <v>78</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A5" s="1">
-        <v>1</v>
+      <c r="A5" s="1" t="s">
+        <v>85</v>
       </c>
       <c r="B5" s="1" t="s">
         <v>25</v>
       </c>
       <c r="C5" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="D5" t="s">
-        <v>78</v>
+        <v>75</v>
       </c>
       <c r="E5">
         <v>1</v>
       </c>
       <c r="F5" t="s">
-        <v>81</v>
+        <v>78</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A6" s="1">
-        <v>2</v>
+      <c r="A6" s="1" t="s">
+        <v>86</v>
       </c>
       <c r="B6" s="1" t="s">
         <v>26</v>
@@ -3349,18 +3275,18 @@
         <v>4</v>
       </c>
       <c r="D6" t="s">
-        <v>78</v>
+        <v>75</v>
       </c>
       <c r="E6">
         <v>1</v>
       </c>
       <c r="F6" t="s">
-        <v>81</v>
+        <v>78</v>
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A7" s="1">
-        <v>2</v>
+      <c r="A7" s="1" t="s">
+        <v>86</v>
       </c>
       <c r="B7" s="1" t="s">
         <v>26</v>
@@ -3369,18 +3295,18 @@
         <v>5</v>
       </c>
       <c r="D7" t="s">
-        <v>78</v>
+        <v>75</v>
       </c>
       <c r="E7">
         <v>1</v>
       </c>
       <c r="F7" t="s">
-        <v>81</v>
+        <v>78</v>
       </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A8" s="1">
-        <v>2</v>
+      <c r="A8" s="1" t="s">
+        <v>86</v>
       </c>
       <c r="B8" s="1" t="s">
         <v>26</v>
@@ -3389,358 +3315,358 @@
         <v>6</v>
       </c>
       <c r="D8" t="s">
-        <v>78</v>
+        <v>75</v>
       </c>
       <c r="E8">
         <v>1</v>
       </c>
       <c r="F8" t="s">
-        <v>81</v>
+        <v>78</v>
       </c>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A9" s="1">
-        <v>2</v>
+      <c r="A9" s="1" t="s">
+        <v>86</v>
       </c>
       <c r="B9" s="1" t="s">
         <v>26</v>
       </c>
       <c r="C9" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="D9" t="s">
-        <v>78</v>
+        <v>75</v>
       </c>
       <c r="E9">
         <v>1</v>
       </c>
       <c r="F9" t="s">
-        <v>81</v>
+        <v>78</v>
       </c>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A10" s="1">
-        <v>3</v>
+      <c r="A10" s="1" t="s">
+        <v>87</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C10" s="1" t="s">
         <v>4</v>
       </c>
       <c r="D10" t="s">
-        <v>78</v>
+        <v>75</v>
       </c>
       <c r="E10">
         <v>1</v>
       </c>
       <c r="F10" t="s">
-        <v>81</v>
+        <v>78</v>
       </c>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A11" s="1">
-        <v>3</v>
+      <c r="A11" s="1" t="s">
+        <v>87</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C11" s="1" t="s">
         <v>6</v>
       </c>
       <c r="D11" t="s">
-        <v>78</v>
+        <v>75</v>
       </c>
       <c r="E11">
         <v>1</v>
       </c>
       <c r="F11" t="s">
-        <v>81</v>
+        <v>78</v>
       </c>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A12" s="1">
-        <v>3</v>
+      <c r="A12" s="1" t="s">
+        <v>87</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C12" s="1" t="s">
         <v>5</v>
       </c>
       <c r="D12" t="s">
-        <v>78</v>
+        <v>75</v>
       </c>
       <c r="E12">
         <v>1</v>
       </c>
       <c r="F12" t="s">
-        <v>81</v>
+        <v>78</v>
       </c>
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A13" s="1">
-        <v>3</v>
+      <c r="A13" s="1" t="s">
+        <v>87</v>
       </c>
       <c r="B13" s="1" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C13" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="D13" t="s">
-        <v>78</v>
+        <v>75</v>
       </c>
       <c r="E13">
         <v>1</v>
       </c>
       <c r="F13" t="s">
-        <v>81</v>
+        <v>78</v>
       </c>
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A14" s="1">
-        <v>4</v>
+      <c r="A14" s="1" t="s">
+        <v>88</v>
       </c>
       <c r="B14" s="1" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="C14" s="1" t="s">
         <v>4</v>
       </c>
       <c r="D14" t="s">
-        <v>78</v>
+        <v>75</v>
       </c>
       <c r="E14">
         <v>1</v>
       </c>
       <c r="F14" t="s">
-        <v>81</v>
+        <v>78</v>
       </c>
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A15" s="1">
-        <v>4</v>
+      <c r="A15" s="1" t="s">
+        <v>88</v>
       </c>
       <c r="B15" s="1" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="C15" s="1" t="s">
         <v>6</v>
       </c>
       <c r="D15" t="s">
-        <v>78</v>
+        <v>75</v>
       </c>
       <c r="E15">
         <v>1</v>
       </c>
       <c r="F15" t="s">
-        <v>81</v>
+        <v>78</v>
       </c>
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A16" s="1">
-        <v>4</v>
+      <c r="A16" s="1" t="s">
+        <v>88</v>
       </c>
       <c r="B16" s="1" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="C16" s="1" t="s">
         <v>5</v>
       </c>
       <c r="D16" t="s">
-        <v>78</v>
+        <v>75</v>
       </c>
       <c r="E16">
         <v>1</v>
       </c>
       <c r="F16" t="s">
-        <v>81</v>
+        <v>78</v>
       </c>
     </row>
     <row r="17" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A17" s="1">
-        <v>4</v>
+      <c r="A17" s="1" t="s">
+        <v>88</v>
       </c>
       <c r="B17" s="1" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="C17" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="D17" t="s">
-        <v>78</v>
+        <v>75</v>
       </c>
       <c r="E17">
         <v>1</v>
       </c>
       <c r="F17" t="s">
-        <v>81</v>
+        <v>78</v>
       </c>
     </row>
     <row r="18" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A18" s="1">
-        <v>5</v>
+      <c r="A18" s="1" t="s">
+        <v>89</v>
       </c>
       <c r="B18" s="1" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="C18" s="1" t="s">
         <v>4</v>
       </c>
       <c r="D18" t="s">
-        <v>78</v>
+        <v>75</v>
       </c>
       <c r="E18">
         <v>1</v>
       </c>
       <c r="F18" t="s">
-        <v>81</v>
+        <v>78</v>
       </c>
     </row>
     <row r="19" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A19" s="1">
-        <v>5</v>
+      <c r="A19" s="1" t="s">
+        <v>89</v>
       </c>
       <c r="B19" s="1" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="C19" s="1" t="s">
         <v>5</v>
       </c>
       <c r="D19" t="s">
-        <v>78</v>
+        <v>75</v>
       </c>
       <c r="E19">
         <v>1</v>
       </c>
       <c r="F19" t="s">
-        <v>81</v>
+        <v>78</v>
       </c>
     </row>
     <row r="20" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A20" s="1">
-        <v>5</v>
+      <c r="A20" s="1" t="s">
+        <v>89</v>
       </c>
       <c r="B20" s="1" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="C20" s="1" t="s">
         <v>6</v>
       </c>
       <c r="D20" t="s">
-        <v>78</v>
+        <v>75</v>
       </c>
       <c r="E20">
         <v>1</v>
       </c>
       <c r="F20" t="s">
-        <v>81</v>
+        <v>78</v>
       </c>
     </row>
     <row r="21" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A21" s="1">
-        <v>5</v>
+      <c r="A21" s="1" t="s">
+        <v>89</v>
       </c>
       <c r="B21" s="1" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="C21" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="D21" t="s">
-        <v>78</v>
+        <v>75</v>
       </c>
       <c r="E21">
         <v>1</v>
       </c>
       <c r="F21" t="s">
-        <v>81</v>
+        <v>78</v>
       </c>
     </row>
     <row r="22" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A22" s="1">
-        <v>6</v>
+      <c r="A22" s="1" t="s">
+        <v>90</v>
       </c>
       <c r="B22" s="1" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="C22" s="1" t="s">
         <v>4</v>
       </c>
       <c r="D22" t="s">
-        <v>78</v>
+        <v>75</v>
       </c>
       <c r="E22">
         <v>1</v>
       </c>
       <c r="F22" t="s">
-        <v>81</v>
+        <v>78</v>
       </c>
     </row>
     <row r="23" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A23" s="1">
-        <v>6</v>
+      <c r="A23" s="1" t="s">
+        <v>90</v>
       </c>
       <c r="B23" s="1" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="C23" s="1" t="s">
         <v>5</v>
       </c>
       <c r="D23" t="s">
-        <v>78</v>
+        <v>75</v>
       </c>
       <c r="E23">
         <v>1</v>
       </c>
       <c r="F23" t="s">
-        <v>81</v>
+        <v>78</v>
       </c>
     </row>
     <row r="24" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A24" s="1">
-        <v>6</v>
+      <c r="A24" s="1" t="s">
+        <v>90</v>
       </c>
       <c r="B24" s="1" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="C24" s="1" t="s">
         <v>6</v>
       </c>
       <c r="D24" t="s">
-        <v>78</v>
+        <v>75</v>
       </c>
       <c r="E24">
         <v>1</v>
       </c>
       <c r="F24" t="s">
-        <v>81</v>
+        <v>78</v>
       </c>
     </row>
     <row r="25" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A25" s="1">
-        <v>6</v>
+      <c r="A25" s="1" t="s">
+        <v>90</v>
       </c>
       <c r="B25" s="1" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="C25" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="D25" t="s">
-        <v>78</v>
+        <v>75</v>
       </c>
       <c r="E25">
         <v>1</v>
       </c>
       <c r="F25" t="s">
-        <v>81</v>
+        <v>78</v>
       </c>
     </row>
     <row r="26" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A26" s="1">
-        <v>7</v>
+      <c r="A26" s="1" t="s">
+        <v>91</v>
       </c>
       <c r="B26" s="1" t="s">
         <v>30</v>
@@ -3749,18 +3675,18 @@
         <v>5</v>
       </c>
       <c r="D26" t="s">
-        <v>79</v>
+        <v>76</v>
       </c>
       <c r="E26">
         <v>2</v>
       </c>
       <c r="F26" t="s">
-        <v>82</v>
+        <v>79</v>
       </c>
     </row>
     <row r="27" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A27" s="1">
-        <v>7</v>
+      <c r="A27" s="1" t="s">
+        <v>91</v>
       </c>
       <c r="B27" s="1" t="s">
         <v>30</v>
@@ -3769,18 +3695,18 @@
         <v>4</v>
       </c>
       <c r="D27" t="s">
-        <v>79</v>
+        <v>76</v>
       </c>
       <c r="E27">
         <v>2</v>
       </c>
       <c r="F27" t="s">
-        <v>82</v>
+        <v>79</v>
       </c>
     </row>
     <row r="28" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A28" s="1">
-        <v>7</v>
+      <c r="A28" s="1" t="s">
+        <v>91</v>
       </c>
       <c r="B28" s="1" t="s">
         <v>30</v>
@@ -3789,18 +3715,18 @@
         <v>6</v>
       </c>
       <c r="D28" t="s">
-        <v>79</v>
+        <v>76</v>
       </c>
       <c r="E28">
         <v>2</v>
       </c>
       <c r="F28" t="s">
-        <v>82</v>
+        <v>79</v>
       </c>
     </row>
     <row r="29" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A29" s="1">
-        <v>8</v>
+      <c r="A29" s="1" t="s">
+        <v>92</v>
       </c>
       <c r="B29" s="1" t="s">
         <v>28</v>
@@ -3809,18 +3735,18 @@
         <v>5</v>
       </c>
       <c r="D29" t="s">
-        <v>79</v>
+        <v>76</v>
       </c>
       <c r="E29">
         <v>2</v>
       </c>
       <c r="F29" t="s">
-        <v>82</v>
+        <v>79</v>
       </c>
     </row>
     <row r="30" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A30" s="1">
-        <v>8</v>
+      <c r="A30" s="1" t="s">
+        <v>92</v>
       </c>
       <c r="B30" s="1" t="s">
         <v>28</v>
@@ -3829,18 +3755,18 @@
         <v>4</v>
       </c>
       <c r="D30" t="s">
-        <v>79</v>
+        <v>76</v>
       </c>
       <c r="E30">
         <v>2</v>
       </c>
       <c r="F30" t="s">
-        <v>82</v>
+        <v>79</v>
       </c>
     </row>
     <row r="31" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A31" s="1">
-        <v>8</v>
+      <c r="A31" s="1" t="s">
+        <v>92</v>
       </c>
       <c r="B31" s="1" t="s">
         <v>28</v>
@@ -3849,839 +3775,1111 @@
         <v>6</v>
       </c>
       <c r="D31" t="s">
-        <v>79</v>
+        <v>76</v>
       </c>
       <c r="E31">
         <v>2</v>
       </c>
       <c r="F31" t="s">
-        <v>82</v>
+        <v>79</v>
       </c>
     </row>
     <row r="32" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A32" s="1">
-        <v>9</v>
+      <c r="A32" s="1" t="s">
+        <v>93</v>
       </c>
       <c r="B32" s="1" t="s">
-        <v>47</v>
-      </c>
-      <c r="C32" s="1"/>
+        <v>46</v>
+      </c>
+      <c r="C32" s="1" t="s">
+        <v>4</v>
+      </c>
       <c r="D32" t="s">
-        <v>78</v>
+        <v>75</v>
       </c>
       <c r="E32">
         <v>1</v>
       </c>
       <c r="F32" t="s">
-        <v>81</v>
+        <v>78</v>
       </c>
     </row>
     <row r="33" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A33" s="1">
-        <v>10</v>
-      </c>
-      <c r="B33" t="s">
+      <c r="A33" s="1" t="s">
+        <v>93</v>
+      </c>
+      <c r="B33" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="C33" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="D33" t="s">
+        <v>75</v>
+      </c>
+      <c r="E33">
+        <v>1</v>
+      </c>
+      <c r="F33" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="34" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A34" s="1" t="s">
+        <v>93</v>
+      </c>
+      <c r="B34" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="C34" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="D34" t="s">
+        <v>75</v>
+      </c>
+      <c r="E34">
+        <v>1</v>
+      </c>
+      <c r="F34" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="35" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A35" s="1" t="s">
+        <v>93</v>
+      </c>
+      <c r="B35" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="C35" t="s">
+        <v>48</v>
+      </c>
+      <c r="D35" t="s">
+        <v>75</v>
+      </c>
+      <c r="E35">
+        <v>1</v>
+      </c>
+      <c r="F35" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="36" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A36" s="1" t="s">
+        <v>94</v>
+      </c>
+      <c r="B36" t="s">
         <v>29</v>
       </c>
-      <c r="C33" s="1"/>
-      <c r="D33" t="s">
+      <c r="C36" s="1"/>
+      <c r="D36" t="s">
+        <v>76</v>
+      </c>
+      <c r="E36">
+        <v>2</v>
+      </c>
+      <c r="F36" t="s">
         <v>79</v>
       </c>
-      <c r="E33">
-        <v>2</v>
-      </c>
-      <c r="F33" t="s">
-        <v>82</v>
-      </c>
-    </row>
-    <row r="34" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A34" s="1">
-        <v>11</v>
-      </c>
-      <c r="B34" s="1" t="s">
+    </row>
+    <row r="37" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A37" s="1" t="s">
+        <v>95</v>
+      </c>
+      <c r="B37" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="C34" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="D34" t="s">
-        <v>78</v>
-      </c>
-      <c r="E34">
-        <v>1</v>
-      </c>
-      <c r="F34" t="s">
-        <v>81</v>
-      </c>
-    </row>
-    <row r="35" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A35" s="1">
-        <v>11</v>
-      </c>
-      <c r="B35" s="1" t="s">
+      <c r="C37" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="D37" t="s">
+        <v>75</v>
+      </c>
+      <c r="E37">
+        <v>1</v>
+      </c>
+      <c r="F37" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="38" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A38" s="1" t="s">
+        <v>95</v>
+      </c>
+      <c r="B38" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="C35" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="D35" t="s">
-        <v>78</v>
-      </c>
-      <c r="E35">
-        <v>1</v>
-      </c>
-      <c r="F35" t="s">
-        <v>81</v>
-      </c>
-    </row>
-    <row r="36" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A36" s="1">
-        <v>11</v>
-      </c>
-      <c r="B36" s="1" t="s">
+      <c r="C38" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="D38" t="s">
+        <v>75</v>
+      </c>
+      <c r="E38">
+        <v>1</v>
+      </c>
+      <c r="F38" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="39" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A39" s="1" t="s">
+        <v>95</v>
+      </c>
+      <c r="B39" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="C36" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="D36" t="s">
-        <v>78</v>
-      </c>
-      <c r="E36">
-        <v>1</v>
-      </c>
-      <c r="F36" t="s">
-        <v>81</v>
-      </c>
-    </row>
-    <row r="37" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A37" s="1">
-        <v>12</v>
-      </c>
-      <c r="B37" s="1" t="s">
+      <c r="C39" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="D39" t="s">
+        <v>75</v>
+      </c>
+      <c r="E39">
+        <v>1</v>
+      </c>
+      <c r="F39" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="40" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A40" s="1" t="s">
+        <v>95</v>
+      </c>
+      <c r="B40" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="C40" t="s">
+        <v>48</v>
+      </c>
+      <c r="D40" t="s">
+        <v>75</v>
+      </c>
+      <c r="E40">
+        <v>1</v>
+      </c>
+      <c r="F40" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="41" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A41" s="1" t="s">
+        <v>96</v>
+      </c>
+      <c r="B41" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="C37" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="D37" t="s">
-        <v>78</v>
-      </c>
-      <c r="E37">
-        <v>1</v>
-      </c>
-      <c r="F37" t="s">
-        <v>81</v>
-      </c>
-    </row>
-    <row r="38" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A38" s="1">
-        <v>12</v>
-      </c>
-      <c r="B38" s="1" t="s">
+      <c r="C41" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="D41" t="s">
+        <v>75</v>
+      </c>
+      <c r="E41">
+        <v>1</v>
+      </c>
+      <c r="F41" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="42" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A42" s="1" t="s">
+        <v>96</v>
+      </c>
+      <c r="B42" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="C38" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="D38" t="s">
-        <v>78</v>
-      </c>
-      <c r="E38">
-        <v>1</v>
-      </c>
-      <c r="F38" t="s">
-        <v>81</v>
-      </c>
-    </row>
-    <row r="39" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A39" s="1">
-        <v>12</v>
-      </c>
-      <c r="B39" s="1" t="s">
+      <c r="C42" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="D42" t="s">
+        <v>75</v>
+      </c>
+      <c r="E42">
+        <v>1</v>
+      </c>
+      <c r="F42" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="43" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A43" s="1" t="s">
+        <v>96</v>
+      </c>
+      <c r="B43" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="C39" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="D39" t="s">
-        <v>78</v>
-      </c>
-      <c r="E39">
-        <v>1</v>
-      </c>
-      <c r="F39" t="s">
-        <v>81</v>
-      </c>
-    </row>
-    <row r="40" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A40" s="1">
-        <v>13</v>
-      </c>
-      <c r="B40" s="1" t="s">
-        <v>41</v>
-      </c>
-      <c r="C40" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="D40" t="s">
-        <v>78</v>
-      </c>
-      <c r="E40">
-        <v>1</v>
-      </c>
-      <c r="F40" t="s">
-        <v>81</v>
-      </c>
-    </row>
-    <row r="41" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A41" s="1">
-        <v>13</v>
-      </c>
-      <c r="B41" s="1" t="s">
-        <v>41</v>
-      </c>
-      <c r="C41" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="D41" t="s">
-        <v>78</v>
-      </c>
-      <c r="E41">
-        <v>1</v>
-      </c>
-      <c r="F41" t="s">
-        <v>81</v>
-      </c>
-    </row>
-    <row r="42" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A42" s="1">
-        <v>13</v>
-      </c>
-      <c r="B42" s="1" t="s">
-        <v>41</v>
-      </c>
-      <c r="C42" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="D42" t="s">
-        <v>78</v>
-      </c>
-      <c r="E42">
-        <v>1</v>
-      </c>
-      <c r="F42" t="s">
-        <v>81</v>
-      </c>
-    </row>
-    <row r="43" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A43" s="1">
-        <v>14</v>
-      </c>
-      <c r="B43" s="1" t="s">
-        <v>65</v>
-      </c>
       <c r="C43" s="1" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="D43" t="s">
-        <v>79</v>
+        <v>75</v>
       </c>
       <c r="E43">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F43" t="s">
-        <v>82</v>
+        <v>78</v>
       </c>
     </row>
     <row r="44" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A44" s="1">
-        <v>14</v>
+      <c r="A44" s="1" t="s">
+        <v>96</v>
       </c>
       <c r="B44" s="1" t="s">
-        <v>65</v>
-      </c>
-      <c r="C44" s="1" t="s">
-        <v>5</v>
+        <v>7</v>
+      </c>
+      <c r="C44" t="s">
+        <v>48</v>
       </c>
       <c r="D44" t="s">
-        <v>79</v>
+        <v>75</v>
       </c>
       <c r="E44">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F44" t="s">
-        <v>82</v>
+        <v>78</v>
       </c>
     </row>
     <row r="45" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A45" s="1">
-        <v>14</v>
+      <c r="A45" s="1" t="s">
+        <v>97</v>
       </c>
       <c r="B45" s="1" t="s">
-        <v>65</v>
+        <v>40</v>
       </c>
       <c r="C45" s="1" t="s">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="D45" t="s">
-        <v>79</v>
+        <v>75</v>
       </c>
       <c r="E45">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F45" t="s">
-        <v>82</v>
+        <v>78</v>
       </c>
     </row>
     <row r="46" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A46" s="1">
-        <v>15</v>
+      <c r="A46" s="1" t="s">
+        <v>97</v>
       </c>
       <c r="B46" s="1" t="s">
-        <v>64</v>
+        <v>40</v>
       </c>
       <c r="C46" s="1" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D46" t="s">
-        <v>79</v>
+        <v>75</v>
       </c>
       <c r="E46">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F46" t="s">
-        <v>82</v>
+        <v>78</v>
       </c>
     </row>
     <row r="47" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A47" s="1">
-        <v>15</v>
+      <c r="A47" s="1" t="s">
+        <v>97</v>
       </c>
       <c r="B47" s="1" t="s">
-        <v>64</v>
+        <v>40</v>
       </c>
       <c r="C47" s="1" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D47" t="s">
-        <v>79</v>
+        <v>75</v>
       </c>
       <c r="E47">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F47" t="s">
-        <v>82</v>
+        <v>78</v>
       </c>
     </row>
     <row r="48" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A48" s="1">
-        <v>15</v>
+      <c r="A48" s="1" t="s">
+        <v>98</v>
       </c>
       <c r="B48" s="1" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="C48" s="1" t="s">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="D48" t="s">
-        <v>79</v>
+        <v>76</v>
       </c>
       <c r="E48">
         <v>2</v>
       </c>
       <c r="F48" t="s">
-        <v>82</v>
+        <v>79</v>
       </c>
     </row>
     <row r="49" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A49" s="1">
-        <v>16</v>
+      <c r="A49" s="1" t="s">
+        <v>98</v>
       </c>
       <c r="B49" s="1" t="s">
+        <v>62</v>
+      </c>
+      <c r="C49" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="D49" t="s">
+        <v>76</v>
+      </c>
+      <c r="E49">
+        <v>2</v>
+      </c>
+      <c r="F49" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="50" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A50" s="1" t="s">
+        <v>98</v>
+      </c>
+      <c r="B50" s="1" t="s">
+        <v>62</v>
+      </c>
+      <c r="C50" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="D50" t="s">
+        <v>76</v>
+      </c>
+      <c r="E50">
+        <v>2</v>
+      </c>
+      <c r="F50" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="51" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A51" s="1" t="s">
+        <v>99</v>
+      </c>
+      <c r="B51" s="1" t="s">
+        <v>61</v>
+      </c>
+      <c r="C51" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="D51" t="s">
+        <v>76</v>
+      </c>
+      <c r="E51">
+        <v>2</v>
+      </c>
+      <c r="F51" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="52" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A52" s="1" t="s">
+        <v>99</v>
+      </c>
+      <c r="B52" s="1" t="s">
+        <v>61</v>
+      </c>
+      <c r="C52" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="D52" t="s">
+        <v>76</v>
+      </c>
+      <c r="E52">
+        <v>2</v>
+      </c>
+      <c r="F52" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="53" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A53" s="1" t="s">
+        <v>99</v>
+      </c>
+      <c r="B53" s="1" t="s">
+        <v>61</v>
+      </c>
+      <c r="C53" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="D53" t="s">
+        <v>76</v>
+      </c>
+      <c r="E53">
+        <v>2</v>
+      </c>
+      <c r="F53" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="54" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A54" s="1" t="s">
+        <v>100</v>
+      </c>
+      <c r="B54" s="1" t="s">
+        <v>60</v>
+      </c>
+      <c r="C54" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="D54" t="s">
+        <v>77</v>
+      </c>
+      <c r="E54">
+        <v>3</v>
+      </c>
+      <c r="F54" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="55" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A55" s="1" t="s">
+        <v>100</v>
+      </c>
+      <c r="B55" s="1" t="s">
+        <v>60</v>
+      </c>
+      <c r="C55" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="D55" t="s">
+        <v>77</v>
+      </c>
+      <c r="E55">
+        <v>3</v>
+      </c>
+      <c r="F55" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="56" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A56" s="1" t="s">
+        <v>100</v>
+      </c>
+      <c r="B56" s="1" t="s">
+        <v>60</v>
+      </c>
+      <c r="C56" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="D56" t="s">
+        <v>77</v>
+      </c>
+      <c r="E56">
+        <v>3</v>
+      </c>
+      <c r="F56" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="57" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A57" s="1" t="s">
+        <v>101</v>
+      </c>
+      <c r="B57" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="C57" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="D57" t="s">
+        <v>75</v>
+      </c>
+      <c r="E57">
+        <v>1</v>
+      </c>
+      <c r="F57" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="58" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A58" s="1" t="s">
+        <v>101</v>
+      </c>
+      <c r="B58" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="C58" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="D58" t="s">
+        <v>75</v>
+      </c>
+      <c r="E58">
+        <v>1</v>
+      </c>
+      <c r="F58" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="59" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A59" s="1" t="s">
+        <v>101</v>
+      </c>
+      <c r="B59" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="C59" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="D59" t="s">
+        <v>75</v>
+      </c>
+      <c r="E59">
+        <v>1</v>
+      </c>
+      <c r="F59" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="60" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A60" s="1" t="s">
+        <v>102</v>
+      </c>
+      <c r="B60" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="C60" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="D60" t="s">
+        <v>75</v>
+      </c>
+      <c r="E60">
+        <v>1</v>
+      </c>
+      <c r="F60" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="61" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A61" s="1" t="s">
+        <v>102</v>
+      </c>
+      <c r="B61" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="C61" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="D61" t="s">
+        <v>75</v>
+      </c>
+      <c r="E61">
+        <v>1</v>
+      </c>
+      <c r="F61" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="62" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A62" s="1" t="s">
+        <v>102</v>
+      </c>
+      <c r="B62" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="C62" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="D62" t="s">
+        <v>75</v>
+      </c>
+      <c r="E62">
+        <v>1</v>
+      </c>
+      <c r="F62" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="63" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A63" s="1" t="s">
+        <v>103</v>
+      </c>
+      <c r="B63" s="1" t="s">
         <v>63</v>
       </c>
-      <c r="C49" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="D49" t="s">
+      <c r="C63" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="D63" t="s">
+        <v>75</v>
+      </c>
+      <c r="E63">
+        <v>1</v>
+      </c>
+      <c r="F63" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="64" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A64" s="1" t="s">
+        <v>103</v>
+      </c>
+      <c r="B64" s="1" t="s">
+        <v>63</v>
+      </c>
+      <c r="C64" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="D64" t="s">
+        <v>75</v>
+      </c>
+      <c r="E64">
+        <v>1</v>
+      </c>
+      <c r="F64" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="65" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A65" s="1" t="s">
+        <v>103</v>
+      </c>
+      <c r="B65" s="1" t="s">
+        <v>63</v>
+      </c>
+      <c r="C65" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="D65" t="s">
+        <v>75</v>
+      </c>
+      <c r="E65">
+        <v>1</v>
+      </c>
+      <c r="F65" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="66" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A66" s="1" t="s">
+        <v>104</v>
+      </c>
+      <c r="B66" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="C66" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="D66" t="s">
+        <v>75</v>
+      </c>
+      <c r="E66">
+        <v>1</v>
+      </c>
+      <c r="F66" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="67" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A67" s="1" t="s">
+        <v>104</v>
+      </c>
+      <c r="B67" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="C67" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="D67" t="s">
+        <v>75</v>
+      </c>
+      <c r="E67">
+        <v>1</v>
+      </c>
+      <c r="F67" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="68" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A68" s="1" t="s">
+        <v>104</v>
+      </c>
+      <c r="B68" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="C68" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="D68" t="s">
+        <v>75</v>
+      </c>
+      <c r="E68">
+        <v>1</v>
+      </c>
+      <c r="F68" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="69" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A69" s="1" t="s">
+        <v>105</v>
+      </c>
+      <c r="B69" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="C69" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="D69" t="s">
+        <v>75</v>
+      </c>
+      <c r="E69">
+        <v>1</v>
+      </c>
+      <c r="F69" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="70" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A70" s="1" t="s">
+        <v>105</v>
+      </c>
+      <c r="B70" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="C70" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="D70" t="s">
+        <v>75</v>
+      </c>
+      <c r="E70">
+        <v>1</v>
+      </c>
+      <c r="F70" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="71" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A71" s="1" t="s">
+        <v>105</v>
+      </c>
+      <c r="B71" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="C71" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="D71" t="s">
+        <v>75</v>
+      </c>
+      <c r="E71">
+        <v>1</v>
+      </c>
+      <c r="F71" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="72" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A72" s="1" t="s">
+        <v>106</v>
+      </c>
+      <c r="B72" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="C72" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="D72" t="s">
+        <v>76</v>
+      </c>
+      <c r="E72">
+        <v>2</v>
+      </c>
+      <c r="F72" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="73" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A73" s="1" t="s">
+        <v>106</v>
+      </c>
+      <c r="B73" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="C73" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="D73" t="s">
+        <v>76</v>
+      </c>
+      <c r="E73">
+        <v>2</v>
+      </c>
+      <c r="F73" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="74" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A74" s="1" t="s">
+        <v>106</v>
+      </c>
+      <c r="B74" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="C74" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="D74" t="s">
+        <v>76</v>
+      </c>
+      <c r="E74">
+        <v>2</v>
+      </c>
+      <c r="F74" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="75" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A75" s="1" t="s">
+        <v>107</v>
+      </c>
+      <c r="B75" s="1" t="s">
+        <v>67</v>
+      </c>
+      <c r="C75" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="D75" t="s">
+        <v>76</v>
+      </c>
+      <c r="E75">
+        <v>2</v>
+      </c>
+      <c r="F75" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="76" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A76" s="1" t="s">
+        <v>107</v>
+      </c>
+      <c r="B76" s="1" t="s">
+        <v>67</v>
+      </c>
+      <c r="C76" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="D76" t="s">
+        <v>76</v>
+      </c>
+      <c r="E76">
+        <v>2</v>
+      </c>
+      <c r="F76" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="77" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A77" s="1" t="s">
+        <v>107</v>
+      </c>
+      <c r="B77" s="1" t="s">
+        <v>67</v>
+      </c>
+      <c r="C77" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="D77" t="s">
+        <v>76</v>
+      </c>
+      <c r="E77">
+        <v>2</v>
+      </c>
+      <c r="F77" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="78" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A78" s="1" t="s">
+        <v>110</v>
+      </c>
+      <c r="B78" s="1" t="s">
+        <v>68</v>
+      </c>
+      <c r="C78" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="D78" t="s">
+        <v>77</v>
+      </c>
+      <c r="E78">
+        <v>3</v>
+      </c>
+      <c r="F78" t="s">
         <v>80</v>
       </c>
-      <c r="E49">
+    </row>
+    <row r="79" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A79" s="1" t="s">
+        <v>110</v>
+      </c>
+      <c r="B79" s="1" t="s">
+        <v>68</v>
+      </c>
+      <c r="C79" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="D79" t="s">
+        <v>77</v>
+      </c>
+      <c r="E79">
         <v>3</v>
       </c>
-      <c r="F49" t="s">
-        <v>83</v>
-      </c>
-    </row>
-    <row r="50" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A50" s="1">
-        <v>16</v>
-      </c>
-      <c r="B50" s="1" t="s">
-        <v>63</v>
-      </c>
-      <c r="C50" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="D50" t="s">
+      <c r="F79" t="s">
         <v>80</v>
       </c>
-      <c r="E50">
+    </row>
+    <row r="80" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A80" s="1" t="s">
+        <v>110</v>
+      </c>
+      <c r="B80" s="1" t="s">
+        <v>68</v>
+      </c>
+      <c r="C80" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="D80" t="s">
+        <v>77</v>
+      </c>
+      <c r="E80">
         <v>3</v>
       </c>
-      <c r="F50" t="s">
-        <v>83</v>
-      </c>
-    </row>
-    <row r="51" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A51" s="1">
-        <v>16</v>
-      </c>
-      <c r="B51" s="1" t="s">
-        <v>63</v>
-      </c>
-      <c r="C51" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="D51" t="s">
+      <c r="F80" t="s">
         <v>80</v>
       </c>
-      <c r="E51">
-        <v>3</v>
-      </c>
-      <c r="F51" t="s">
-        <v>83</v>
-      </c>
-    </row>
-    <row r="52" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A52" s="1">
-        <v>17</v>
-      </c>
-      <c r="B52" s="1" t="s">
-        <v>35</v>
-      </c>
-      <c r="D52" t="s">
-        <v>78</v>
-      </c>
-      <c r="E52">
-        <v>1</v>
-      </c>
-      <c r="F52" t="s">
-        <v>81</v>
-      </c>
-    </row>
-    <row r="53" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A53" s="1">
-        <v>18</v>
-      </c>
-      <c r="B53" s="1" t="s">
-        <v>34</v>
-      </c>
-      <c r="D53" t="s">
-        <v>78</v>
-      </c>
-      <c r="E53">
-        <v>1</v>
-      </c>
-      <c r="F53" t="s">
-        <v>81</v>
-      </c>
-    </row>
-    <row r="54" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A54" s="1">
-        <v>19</v>
-      </c>
-      <c r="B54" s="1" t="s">
-        <v>66</v>
-      </c>
-      <c r="C54" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="D54" t="s">
-        <v>78</v>
-      </c>
-      <c r="E54">
-        <v>1</v>
-      </c>
-      <c r="F54" t="s">
-        <v>81</v>
-      </c>
-    </row>
-    <row r="55" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A55" s="1">
-        <v>19</v>
-      </c>
-      <c r="B55" s="1" t="s">
-        <v>66</v>
-      </c>
-      <c r="C55" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="D55" t="s">
-        <v>78</v>
-      </c>
-      <c r="E55">
-        <v>1</v>
-      </c>
-      <c r="F55" t="s">
-        <v>81</v>
-      </c>
-    </row>
-    <row r="56" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A56" s="1">
-        <v>19</v>
-      </c>
-      <c r="B56" s="1" t="s">
-        <v>66</v>
-      </c>
-      <c r="C56" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="D56" t="s">
-        <v>78</v>
-      </c>
-      <c r="E56">
-        <v>1</v>
-      </c>
-      <c r="F56" t="s">
-        <v>81</v>
-      </c>
-    </row>
-    <row r="57" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A57" s="1">
-        <v>20</v>
-      </c>
-      <c r="B57" s="1" t="s">
-        <v>67</v>
-      </c>
-      <c r="C57" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="D57" t="s">
-        <v>78</v>
-      </c>
-      <c r="E57">
-        <v>1</v>
-      </c>
-      <c r="F57" t="s">
-        <v>81</v>
-      </c>
-    </row>
-    <row r="58" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A58" s="1">
-        <v>20</v>
-      </c>
-      <c r="B58" s="1" t="s">
-        <v>67</v>
-      </c>
-      <c r="C58" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="D58" t="s">
-        <v>78</v>
-      </c>
-      <c r="E58">
-        <v>1</v>
-      </c>
-      <c r="F58" t="s">
-        <v>81</v>
-      </c>
-    </row>
-    <row r="59" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A59" s="1">
-        <v>20</v>
-      </c>
-      <c r="B59" s="1" t="s">
-        <v>67</v>
-      </c>
-      <c r="C59" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="D59" t="s">
-        <v>78</v>
-      </c>
-      <c r="E59">
-        <v>1</v>
-      </c>
-      <c r="F59" t="s">
-        <v>81</v>
-      </c>
-    </row>
-    <row r="60" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A60" s="1">
-        <v>21</v>
-      </c>
-      <c r="B60" s="1" t="s">
-        <v>68</v>
-      </c>
-      <c r="C60" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="D60" t="s">
-        <v>78</v>
-      </c>
-      <c r="E60">
-        <v>1</v>
-      </c>
-      <c r="F60" t="s">
-        <v>81</v>
-      </c>
-    </row>
-    <row r="61" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A61" s="1">
-        <v>21</v>
-      </c>
-      <c r="B61" s="1" t="s">
-        <v>68</v>
-      </c>
-      <c r="C61" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="D61" t="s">
-        <v>78</v>
-      </c>
-      <c r="E61">
-        <v>1</v>
-      </c>
-      <c r="F61" t="s">
-        <v>81</v>
-      </c>
-    </row>
-    <row r="62" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A62" s="1">
-        <v>21</v>
-      </c>
-      <c r="B62" s="1" t="s">
-        <v>68</v>
-      </c>
-      <c r="C62" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="D62" t="s">
-        <v>78</v>
-      </c>
-      <c r="E62">
-        <v>1</v>
-      </c>
-      <c r="F62" t="s">
-        <v>81</v>
-      </c>
-    </row>
-    <row r="63" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A63" s="1">
-        <v>22</v>
-      </c>
-      <c r="B63" s="1" t="s">
+    </row>
+    <row r="81" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A81" s="1" t="s">
+        <v>108</v>
+      </c>
+      <c r="B81" s="1" t="s">
         <v>69</v>
       </c>
-      <c r="C63" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="D63" t="s">
-        <v>79</v>
-      </c>
-      <c r="E63">
-        <v>2</v>
-      </c>
-      <c r="F63" t="s">
-        <v>82</v>
-      </c>
-    </row>
-    <row r="64" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A64" s="1">
-        <v>22</v>
-      </c>
-      <c r="B64" s="1" t="s">
+      <c r="C81" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="D81" t="s">
+        <v>75</v>
+      </c>
+      <c r="E81">
+        <v>1</v>
+      </c>
+      <c r="F81" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="82" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A82" s="1" t="s">
+        <v>108</v>
+      </c>
+      <c r="B82" s="1" t="s">
         <v>69</v>
       </c>
-      <c r="C64" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="D64" t="s">
-        <v>79</v>
-      </c>
-      <c r="E64">
-        <v>2</v>
-      </c>
-      <c r="F64" t="s">
-        <v>82</v>
-      </c>
-    </row>
-    <row r="65" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A65" s="1">
-        <v>22</v>
-      </c>
-      <c r="B65" s="1" t="s">
+      <c r="C82" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="D82" t="s">
+        <v>75</v>
+      </c>
+      <c r="E82">
+        <v>1</v>
+      </c>
+      <c r="F82" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="83" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A83" s="1" t="s">
+        <v>108</v>
+      </c>
+      <c r="B83" s="1" t="s">
         <v>69</v>
       </c>
-      <c r="C65" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="D65" t="s">
-        <v>79</v>
-      </c>
-      <c r="E65">
-        <v>2</v>
-      </c>
-      <c r="F65" t="s">
-        <v>82</v>
-      </c>
-    </row>
-    <row r="66" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A66" s="1">
-        <v>23</v>
-      </c>
-      <c r="B66" s="1" t="s">
+      <c r="C83" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="D83" t="s">
+        <v>75</v>
+      </c>
+      <c r="E83">
+        <v>1</v>
+      </c>
+      <c r="F83" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="84" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A84" s="1" t="s">
+        <v>109</v>
+      </c>
+      <c r="B84" s="1" t="s">
         <v>70</v>
       </c>
-      <c r="C66" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="D66" t="s">
-        <v>79</v>
-      </c>
-      <c r="E66">
-        <v>2</v>
-      </c>
-      <c r="F66" t="s">
-        <v>82</v>
-      </c>
-    </row>
-    <row r="67" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A67" s="1">
-        <v>23</v>
-      </c>
-      <c r="B67" s="1" t="s">
+      <c r="C84" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="D84" t="s">
+        <v>75</v>
+      </c>
+      <c r="E84">
+        <v>1</v>
+      </c>
+      <c r="F84" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="85" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A85" s="1" t="s">
+        <v>109</v>
+      </c>
+      <c r="B85" s="1" t="s">
         <v>70</v>
       </c>
-      <c r="C67" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="D67" t="s">
-        <v>79</v>
-      </c>
-      <c r="E67">
-        <v>2</v>
-      </c>
-      <c r="F67" t="s">
-        <v>82</v>
-      </c>
-    </row>
-    <row r="68" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A68" s="1">
-        <v>23</v>
-      </c>
-      <c r="B68" s="1" t="s">
+      <c r="C85" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="D85" t="s">
+        <v>75</v>
+      </c>
+      <c r="E85">
+        <v>1</v>
+      </c>
+      <c r="F85" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="86" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A86" s="1" t="s">
+        <v>109</v>
+      </c>
+      <c r="B86" s="1" t="s">
         <v>70</v>
       </c>
-      <c r="C68" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="D68" t="s">
-        <v>79</v>
-      </c>
-      <c r="E68">
-        <v>2</v>
-      </c>
-      <c r="F68" t="s">
-        <v>82</v>
-      </c>
-    </row>
-    <row r="69" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A69" s="1">
-        <v>24</v>
-      </c>
-      <c r="B69" s="1" t="s">
-        <v>71</v>
-      </c>
-      <c r="C69" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="D69" t="s">
-        <v>80</v>
-      </c>
-      <c r="E69">
-        <v>3</v>
-      </c>
-      <c r="F69" t="s">
-        <v>83</v>
-      </c>
-    </row>
-    <row r="70" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A70" s="1">
-        <v>24</v>
-      </c>
-      <c r="B70" s="1" t="s">
-        <v>71</v>
-      </c>
-      <c r="C70" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="D70" t="s">
-        <v>80</v>
-      </c>
-      <c r="E70">
-        <v>3</v>
-      </c>
-      <c r="F70" t="s">
-        <v>83</v>
-      </c>
-    </row>
-    <row r="71" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A71" s="1">
-        <v>24</v>
-      </c>
-      <c r="B71" s="1" t="s">
-        <v>71</v>
-      </c>
-      <c r="C71" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="D71" t="s">
-        <v>80</v>
-      </c>
-      <c r="E71">
-        <v>3</v>
-      </c>
-      <c r="F71" t="s">
-        <v>83</v>
-      </c>
-    </row>
-    <row r="72" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A72" s="1">
-        <v>25</v>
-      </c>
-      <c r="B72" s="1" t="s">
-        <v>72</v>
-      </c>
-      <c r="C72" s="1"/>
-      <c r="D72" t="s">
-        <v>78</v>
-      </c>
-      <c r="E72">
-        <v>1</v>
-      </c>
-      <c r="F72" t="s">
-        <v>81</v>
-      </c>
-    </row>
-    <row r="73" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A73" s="1">
-        <v>26</v>
-      </c>
-      <c r="B73" s="1" t="s">
-        <v>73</v>
-      </c>
-      <c r="C73" s="1"/>
-      <c r="D73" t="s">
-        <v>78</v>
-      </c>
-      <c r="E73">
-        <v>1</v>
-      </c>
-      <c r="F73" t="s">
-        <v>81</v>
+      <c r="C86" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="D86" t="s">
+        <v>75</v>
+      </c>
+      <c r="E86">
+        <v>1</v>
+      </c>
+      <c r="F86" t="s">
+        <v>78</v>
       </c>
     </row>
   </sheetData>

</xml_diff>